<commit_message>
Done with day 14
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="129">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -421,7 +421,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -497,13 +497,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <u val="single"/>
-      <sz val="13"/>
-      <color theme="10"/>
-      <name val="ComicShannsMono Nerd Font"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="8">
@@ -617,100 +610,100 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -718,15 +711,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -734,15 +727,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -750,19 +743,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -770,19 +759,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1925,7 +1906,7 @@
       <c r="D12" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="34" t="s">
+      <c r="E12" s="24" t="s">
         <v>89</v>
       </c>
       <c r="F12" s="23" t="s">
@@ -1985,11 +1966,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="18" width="11.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="18" width="94.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="18" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="19" width="9.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="19" width="9.79"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="8" style="18" width="8.88"/>
   </cols>
   <sheetData>
-    <row r="1" s="35" customFormat="true" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" s="34" customFormat="true" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
@@ -2032,42 +2013,42 @@
       <c r="G2" s="25"/>
     </row>
     <row r="3" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="36" t="n">
+      <c r="A3" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="35" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="36" t="s">
+      <c r="C3" s="35" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="36" t="s">
+      <c r="D3" s="35" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="E3" s="36" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="36"/>
-      <c r="G3" s="36"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
     </row>
     <row r="4" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="38" t="n">
+      <c r="A4" s="37" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="38" t="s">
+      <c r="B4" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="38" t="s">
+      <c r="C4" s="37" t="s">
         <v>95</v>
       </c>
-      <c r="D4" s="38" t="s">
+      <c r="D4" s="37" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="39" t="s">
+      <c r="E4" s="38" t="s">
         <v>96</v>
       </c>
-      <c r="F4" s="38"/>
-      <c r="G4" s="38"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="37"/>
     </row>
     <row r="5" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="n">
@@ -2089,23 +2070,23 @@
       <c r="G5" s="25"/>
     </row>
     <row r="6" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="40" t="n">
+      <c r="A6" s="31" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="40" t="s">
+      <c r="C6" s="31" t="s">
         <v>99</v>
       </c>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="31" t="s">
         <v>34</v>
       </c>
       <c r="E6" s="32" t="s">
         <v>100</v>
       </c>
-      <c r="F6" s="40"/>
-      <c r="G6" s="40"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
     </row>
     <row r="7" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="n">
@@ -2123,8 +2104,12 @@
       <c r="E7" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="F7" s="23"/>
-      <c r="G7" s="25"/>
+      <c r="F7" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="25" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="n">
@@ -2165,8 +2150,12 @@
       <c r="E9" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="25"/>
+      <c r="F9" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="25" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="n">
@@ -2181,7 +2170,7 @@
       <c r="D10" s="23" t="s">
         <v>108</v>
       </c>
-      <c r="E10" s="41" t="s">
+      <c r="E10" s="24" t="s">
         <v>109</v>
       </c>
       <c r="F10" s="23"/>
@@ -2249,61 +2238,61 @@
       <c r="G13" s="25"/>
     </row>
     <row r="14" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="40" t="n">
+      <c r="A14" s="31" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="40" t="s">
+      <c r="B14" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="C14" s="40" t="s">
+      <c r="C14" s="31" t="s">
         <v>116</v>
       </c>
-      <c r="D14" s="40" t="s">
+      <c r="D14" s="31" t="s">
         <v>34</v>
       </c>
       <c r="E14" s="32" t="s">
         <v>117</v>
       </c>
-      <c r="F14" s="40"/>
-      <c r="G14" s="40"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
     </row>
     <row r="15" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="40" t="n">
+      <c r="A15" s="31" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="40" t="s">
+      <c r="B15" s="31" t="s">
         <v>90</v>
       </c>
-      <c r="C15" s="40" t="s">
+      <c r="C15" s="31" t="s">
         <v>118</v>
       </c>
-      <c r="D15" s="40" t="s">
+      <c r="D15" s="31" t="s">
         <v>34</v>
       </c>
       <c r="E15" s="32" t="s">
         <v>119</v>
       </c>
-      <c r="F15" s="40"/>
-      <c r="G15" s="40"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="31"/>
     </row>
     <row r="16" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="40" t="n">
+      <c r="A16" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="35" t="s">
         <v>90</v>
       </c>
-      <c r="C16" s="36" t="s">
+      <c r="C16" s="35" t="s">
         <v>120</v>
       </c>
-      <c r="D16" s="36" t="s">
+      <c r="D16" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="37" t="s">
+      <c r="E16" s="36" t="s">
         <v>121</v>
       </c>
-      <c r="F16" s="36"/>
-      <c r="G16" s="40"/>
+      <c r="F16" s="35"/>
+      <c r="G16" s="31"/>
     </row>
     <row r="17" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="n">

</xml_diff>

<commit_message>
Done with day 15
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="129">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -1663,7 +1663,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
@@ -1709,7 +1709,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
@@ -1732,7 +1732,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
@@ -1755,7 +1755,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <v>5</v>
       </c>
@@ -1778,7 +1778,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
         <v>6</v>
       </c>
@@ -1801,7 +1801,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
         <v>7</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>8</v>
       </c>
@@ -1847,7 +1847,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>9</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>10</v>
       </c>
@@ -1893,7 +1893,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>11</v>
       </c>
@@ -1993,7 +1993,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="23" t="n">
         <v>1</v>
       </c>
@@ -2009,10 +2009,14 @@
       <c r="E2" s="24" t="s">
         <v>92</v>
       </c>
-      <c r="F2" s="23"/>
-      <c r="G2" s="25"/>
-    </row>
-    <row r="3" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F2" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="25" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="35" t="n">
         <v>2</v>
       </c>
@@ -2031,7 +2035,7 @@
       <c r="F3" s="35"/>
       <c r="G3" s="35"/>
     </row>
-    <row r="4" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="37" t="n">
         <v>3</v>
       </c>
@@ -2050,7 +2054,7 @@
       <c r="F4" s="37"/>
       <c r="G4" s="37"/>
     </row>
-    <row r="5" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="23" t="n">
         <v>4</v>
       </c>
@@ -2069,7 +2073,7 @@
       <c r="F5" s="23"/>
       <c r="G5" s="25"/>
     </row>
-    <row r="6" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="31" t="n">
         <v>5</v>
       </c>
@@ -2088,7 +2092,7 @@
       <c r="F6" s="31"/>
       <c r="G6" s="31"/>
     </row>
-    <row r="7" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="23" t="n">
         <v>6</v>
       </c>
@@ -2111,7 +2115,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="n">
         <v>7</v>
       </c>
@@ -2134,7 +2138,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="n">
         <v>8</v>
       </c>
@@ -2157,7 +2161,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="n">
         <v>9</v>
       </c>
@@ -2176,7 +2180,7 @@
       <c r="F10" s="23"/>
       <c r="G10" s="25"/>
     </row>
-    <row r="11" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="n">
         <v>10</v>
       </c>
@@ -2195,7 +2199,7 @@
       <c r="F11" s="23"/>
       <c r="G11" s="25"/>
     </row>
-    <row r="12" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="n">
         <v>11</v>
       </c>
@@ -2218,7 +2222,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="23" t="n">
         <v>12</v>
       </c>
@@ -2237,7 +2241,7 @@
       <c r="F13" s="23"/>
       <c r="G13" s="25"/>
     </row>
-    <row r="14" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="31" t="n">
         <v>13</v>
       </c>
@@ -2256,7 +2260,7 @@
       <c r="F14" s="31"/>
       <c r="G14" s="31"/>
     </row>
-    <row r="15" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="31" t="n">
         <v>14</v>
       </c>
@@ -2275,7 +2279,7 @@
       <c r="F15" s="31"/>
       <c r="G15" s="31"/>
     </row>
-    <row r="16" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="31" t="n">
         <v>15</v>
       </c>
@@ -2294,7 +2298,7 @@
       <c r="F16" s="35"/>
       <c r="G16" s="31"/>
     </row>
-    <row r="17" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="23" t="n">
         <v>16</v>
       </c>
@@ -2317,7 +2321,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="23" t="n">
         <v>17</v>
       </c>
@@ -2340,7 +2344,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="23" t="n">
         <v>18</v>
       </c>
@@ -2359,7 +2363,7 @@
       <c r="F19" s="23"/>
       <c r="G19" s="25"/>
     </row>
-    <row r="20" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="23" t="n">
         <v>19</v>
       </c>

</xml_diff>

<commit_message>
Done with day 16
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="129">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -2196,8 +2196,12 @@
       <c r="E11" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="23"/>
-      <c r="G11" s="25"/>
+      <c r="F11" s="23" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="25" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="n">

</xml_diff>

<commit_message>
Done with day 17
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="129">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -421,7 +421,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -496,6 +496,44 @@
       <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="13"/>
+      <color theme="10"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color rgb="FF000000"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -610,7 +648,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="46">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -747,23 +785,51 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="7" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="7" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1970,421 +2036,425 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="8" style="18" width="8.88"/>
   </cols>
   <sheetData>
-    <row r="1" s="34" customFormat="true" ht="19.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
+    <row r="1" s="36" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="34" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="34" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="20" t="s">
+      <c r="E1" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="35" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="n">
+    <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="37" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="23" t="s">
+      <c r="D2" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="E2" s="38" t="s">
         <v>92</v>
       </c>
-      <c r="F2" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="25" t="n">
+      <c r="F2" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="39" t="n">
         <v>15</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="35" t="n">
+    <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="40" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="35" t="s">
+      <c r="B3" s="40" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="35" t="s">
+      <c r="C3" s="40" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="35" t="s">
+      <c r="D3" s="40" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="36" t="s">
+      <c r="E3" s="41" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="35"/>
-      <c r="G3" s="35"/>
-    </row>
-    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="37" t="n">
+      <c r="F3" s="40"/>
+      <c r="G3" s="40"/>
+    </row>
+    <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="42" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="37" t="s">
+      <c r="B4" s="42" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="37" t="s">
+      <c r="C4" s="42" t="s">
         <v>95</v>
       </c>
-      <c r="D4" s="37" t="s">
+      <c r="D4" s="42" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="38" t="s">
+      <c r="E4" s="43" t="s">
         <v>96</v>
       </c>
-      <c r="F4" s="37"/>
-      <c r="G4" s="37"/>
-    </row>
-    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="n">
+      <c r="F4" s="42"/>
+      <c r="G4" s="42"/>
+    </row>
+    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="37" t="s">
         <v>97</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="38" t="s">
         <v>98</v>
       </c>
-      <c r="F5" s="23"/>
-      <c r="G5" s="25"/>
-    </row>
-    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="n">
+      <c r="F5" s="37"/>
+      <c r="G5" s="39"/>
+    </row>
+    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="44" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="31" t="s">
+      <c r="B6" s="44" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="31" t="s">
+      <c r="C6" s="44" t="s">
         <v>99</v>
       </c>
-      <c r="D6" s="31" t="s">
+      <c r="D6" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="32" t="s">
+      <c r="E6" s="45" t="s">
         <v>100</v>
       </c>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-    </row>
-    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="n">
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+    </row>
+    <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="37" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="23" t="s">
+      <c r="B7" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="37" t="s">
         <v>101</v>
       </c>
-      <c r="D7" s="23" t="s">
+      <c r="D7" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="24" t="s">
+      <c r="E7" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="F7" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="25" t="n">
+      <c r="F7" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="39" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="23" t="s">
+    <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="D8" s="23" t="s">
+      <c r="D8" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="24" t="s">
+      <c r="E8" s="38" t="s">
         <v>104</v>
       </c>
-      <c r="F8" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="25" t="n">
+      <c r="F8" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="39" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="23" t="n">
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="37" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="23" t="s">
+      <c r="B9" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C9" s="23" t="s">
+      <c r="C9" s="37" t="s">
         <v>105</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="24" t="s">
+      <c r="E9" s="38" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="25" t="n">
+      <c r="F9" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="39" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="23" t="n">
+    <row r="10" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="37" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="23" t="s">
+      <c r="B10" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C10" s="37" t="s">
         <v>107</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="D10" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="38" t="s">
         <v>109</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="25"/>
-    </row>
-    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="23" t="n">
+      <c r="F10" s="37"/>
+      <c r="G10" s="39"/>
+    </row>
+    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="37" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C11" s="23" t="s">
+      <c r="C11" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="D11" s="23" t="s">
+      <c r="D11" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="24" t="s">
+      <c r="E11" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="25" t="n">
+      <c r="F11" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="39" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="23" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="23" t="s">
+    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="37" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="D12" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="24" t="s">
+      <c r="E12" s="38" t="s">
         <v>113</v>
       </c>
-      <c r="F12" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" s="25" t="n">
+      <c r="F12" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="39" t="n">
         <v>14</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="23" t="n">
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="37" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="23" t="s">
+      <c r="B13" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="37" t="s">
         <v>114</v>
       </c>
-      <c r="D13" s="23" t="s">
+      <c r="D13" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="24" t="s">
+      <c r="E13" s="38" t="s">
         <v>115</v>
       </c>
-      <c r="F13" s="23"/>
-      <c r="G13" s="25"/>
-    </row>
-    <row r="14" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="31" t="n">
+      <c r="F13" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="39" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="44" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="31" t="s">
+      <c r="B14" s="44" t="s">
         <v>90</v>
       </c>
-      <c r="C14" s="31" t="s">
+      <c r="C14" s="44" t="s">
         <v>116</v>
       </c>
-      <c r="D14" s="31" t="s">
+      <c r="D14" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="E14" s="32" t="s">
+      <c r="E14" s="45" t="s">
         <v>117</v>
       </c>
-      <c r="F14" s="31"/>
-      <c r="G14" s="31"/>
-    </row>
-    <row r="15" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="31" t="n">
+      <c r="F14" s="44"/>
+      <c r="G14" s="44"/>
+    </row>
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="44" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="31" t="s">
+      <c r="B15" s="44" t="s">
         <v>90</v>
       </c>
-      <c r="C15" s="31" t="s">
+      <c r="C15" s="44" t="s">
         <v>118</v>
       </c>
-      <c r="D15" s="31" t="s">
+      <c r="D15" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="E15" s="32" t="s">
+      <c r="E15" s="45" t="s">
         <v>119</v>
       </c>
-      <c r="F15" s="31"/>
-      <c r="G15" s="31"/>
-    </row>
-    <row r="16" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="31" t="n">
+      <c r="F15" s="44"/>
+      <c r="G15" s="44"/>
+    </row>
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="44" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="35" t="s">
+      <c r="B16" s="40" t="s">
         <v>90</v>
       </c>
-      <c r="C16" s="35" t="s">
+      <c r="C16" s="40" t="s">
         <v>120</v>
       </c>
-      <c r="D16" s="35" t="s">
+      <c r="D16" s="40" t="s">
         <v>43</v>
       </c>
-      <c r="E16" s="36" t="s">
+      <c r="E16" s="41" t="s">
         <v>121</v>
       </c>
-      <c r="F16" s="35"/>
-      <c r="G16" s="31"/>
-    </row>
-    <row r="17" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23" t="n">
+      <c r="F16" s="40"/>
+      <c r="G16" s="44"/>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="37" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="23" t="s">
+      <c r="B17" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="23" t="s">
+      <c r="C17" s="37" t="s">
         <v>122</v>
       </c>
-      <c r="D17" s="23" t="s">
+      <c r="D17" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="24" t="s">
+      <c r="E17" s="38" t="s">
         <v>123</v>
       </c>
-      <c r="F17" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="G17" s="25" t="n">
+      <c r="F17" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="39" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="n">
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="37" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="37" t="s">
         <v>124</v>
       </c>
-      <c r="D18" s="23" t="s">
+      <c r="D18" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="24" t="s">
+      <c r="E18" s="38" t="s">
         <v>125</v>
       </c>
-      <c r="F18" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="G18" s="25" t="n">
+      <c r="F18" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="39" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="n">
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="37" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C19" s="23" t="s">
+      <c r="C19" s="37" t="s">
         <v>126</v>
       </c>
-      <c r="D19" s="23" t="s">
+      <c r="D19" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="24" t="s">
+      <c r="E19" s="38" t="s">
         <v>92</v>
       </c>
-      <c r="F19" s="23"/>
-      <c r="G19" s="25"/>
-    </row>
-    <row r="20" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="23" t="n">
+      <c r="F19" s="37"/>
+      <c r="G19" s="39"/>
+    </row>
+    <row r="20" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="37" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C20" s="23" t="s">
+      <c r="C20" s="37" t="s">
         <v>127</v>
       </c>
-      <c r="D20" s="23" t="s">
+      <c r="D20" s="37" t="s">
         <v>128</v>
       </c>
-      <c r="E20" s="24" t="s">
+      <c r="E20" s="38" t="s">
         <v>102</v>
       </c>
-      <c r="F20" s="23"/>
-      <c r="G20" s="25"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="39"/>
     </row>
     <row r="21" s="18" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="22" s="18" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Done with day 18
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="130">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -321,6 +321,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/longest-repeating-character-replacement/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes</t>
   </si>
   <si>
     <t xml:space="preserve">76. Minimum Window Substring</t>
@@ -499,6 +502,13 @@
       <charset val="1"/>
     </font>
     <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Comic Sans MS"/>
+      <family val="4"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
       <sz val="13"/>
       <color theme="1"/>
@@ -510,13 +520,6 @@
       <b val="true"/>
       <sz val="13"/>
       <color rgb="FF000000"/>
-      <name val="Comic Sans MS"/>
-      <family val="4"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="13"/>
-      <color theme="1"/>
       <name val="Comic Sans MS"/>
       <family val="4"/>
       <charset val="1"/>
@@ -648,7 +651,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="48">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -785,19 +788,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -809,7 +820,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -817,7 +828,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -825,7 +836,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2026,441 +2037,445 @@
   <dimension ref="A1:G25"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="19.5" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="18" width="5.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="18" width="18.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="18" width="65.44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="18" width="11.89"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="18" width="94.32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="18" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="19" width="9.79"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="8" style="18" width="8.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="34" width="5.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="34" width="18.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="34" width="65.44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="34" width="11.89"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="34" width="94.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="34" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="35" width="9.79"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="8" style="34" width="8.88"/>
   </cols>
   <sheetData>
-    <row r="1" s="36" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="34" t="s">
+    <row r="1" s="38" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34" t="s">
+      <c r="B1" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="36" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="E1" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="34" t="s">
+      <c r="F1" s="36" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="35" t="s">
+      <c r="G1" s="37" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="37" t="n">
+      <c r="A2" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="39" t="s">
         <v>90</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="39" t="s">
         <v>91</v>
       </c>
-      <c r="D2" s="37" t="s">
+      <c r="D2" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="38" t="s">
+      <c r="E2" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="F2" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="G2" s="39" t="n">
+      <c r="F2" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="41" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="40" t="n">
+      <c r="A3" s="42" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="42" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="40" t="s">
+      <c r="C3" s="42" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="42" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="43" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
+      <c r="F3" s="42"/>
+      <c r="G3" s="42"/>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="42" t="n">
+      <c r="A4" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="42" t="s">
+      <c r="B4" s="44" t="s">
         <v>90</v>
       </c>
-      <c r="C4" s="42" t="s">
+      <c r="C4" s="44" t="s">
         <v>95</v>
       </c>
-      <c r="D4" s="42" t="s">
+      <c r="D4" s="44" t="s">
         <v>43</v>
       </c>
-      <c r="E4" s="43" t="s">
+      <c r="E4" s="45" t="s">
         <v>96</v>
       </c>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
+      <c r="F4" s="44"/>
+      <c r="G4" s="44"/>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="37" t="n">
+      <c r="A5" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="37" t="s">
+      <c r="B5" s="39" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="37" t="s">
+      <c r="C5" s="39" t="s">
         <v>97</v>
       </c>
-      <c r="D5" s="37" t="s">
+      <c r="D5" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="38" t="s">
+      <c r="E5" s="40" t="s">
         <v>98</v>
       </c>
-      <c r="F5" s="37"/>
-      <c r="G5" s="39"/>
+      <c r="F5" s="39" t="s">
+        <v>99</v>
+      </c>
+      <c r="G5" s="41" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="44" t="n">
+      <c r="A6" s="46" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="44" t="s">
+      <c r="B6" s="46" t="s">
         <v>90</v>
       </c>
-      <c r="C6" s="44" t="s">
-        <v>99</v>
-      </c>
-      <c r="D6" s="44" t="s">
+      <c r="C6" s="46" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" s="46" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="45" t="s">
-        <v>100</v>
-      </c>
-      <c r="F6" s="44"/>
-      <c r="G6" s="44"/>
+      <c r="E6" s="47" t="s">
+        <v>101</v>
+      </c>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="37" t="n">
+      <c r="A7" s="39" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="37" t="s">
+      <c r="B7" s="39" t="s">
         <v>90</v>
       </c>
-      <c r="C7" s="37" t="s">
-        <v>101</v>
-      </c>
-      <c r="D7" s="37" t="s">
+      <c r="C7" s="39" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="38" t="s">
-        <v>102</v>
-      </c>
-      <c r="F7" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="39" t="n">
+      <c r="E7" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="F7" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="41" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="37" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="37" t="s">
+      <c r="A8" s="39" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="39" t="s">
         <v>90</v>
       </c>
-      <c r="C8" s="37" t="s">
+      <c r="C8" s="39" t="s">
+        <v>104</v>
+      </c>
+      <c r="D8" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="F8" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="41" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="39" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" s="39" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="39" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="40" t="s">
+        <v>107</v>
+      </c>
+      <c r="F9" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" s="41" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="39" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="C10" s="39" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="39" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="40" t="s">
+        <v>110</v>
+      </c>
+      <c r="F10" s="39"/>
+      <c r="G10" s="41"/>
+    </row>
+    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="39" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11" s="39" t="s">
+        <v>111</v>
+      </c>
+      <c r="D11" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="F11" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="41" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="39" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12" s="39" t="s">
+        <v>113</v>
+      </c>
+      <c r="D12" s="39" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="40" t="s">
+        <v>114</v>
+      </c>
+      <c r="F12" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="41" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="39" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="C13" s="39" t="s">
+        <v>115</v>
+      </c>
+      <c r="D13" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="40" t="s">
+        <v>116</v>
+      </c>
+      <c r="F13" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="41" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="46" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>117</v>
+      </c>
+      <c r="D14" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="47" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" s="46"/>
+      <c r="G14" s="46"/>
+    </row>
+    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="46" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="46" t="s">
+        <v>90</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>119</v>
+      </c>
+      <c r="D15" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="47" t="s">
+        <v>120</v>
+      </c>
+      <c r="F15" s="46"/>
+      <c r="G15" s="46"/>
+    </row>
+    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="46" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="42" t="s">
+        <v>90</v>
+      </c>
+      <c r="C16" s="42" t="s">
+        <v>121</v>
+      </c>
+      <c r="D16" s="42" t="s">
+        <v>43</v>
+      </c>
+      <c r="E16" s="43" t="s">
+        <v>122</v>
+      </c>
+      <c r="F16" s="42"/>
+      <c r="G16" s="46"/>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="39" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" s="39" t="s">
+        <v>123</v>
+      </c>
+      <c r="D17" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" s="40" t="s">
+        <v>124</v>
+      </c>
+      <c r="F17" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="41" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="39" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="C18" s="39" t="s">
+        <v>125</v>
+      </c>
+      <c r="D18" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="F18" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="41" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="39" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="C19" s="39" t="s">
+        <v>127</v>
+      </c>
+      <c r="D19" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="40" t="s">
+        <v>92</v>
+      </c>
+      <c r="F19" s="39"/>
+      <c r="G19" s="41"/>
+    </row>
+    <row r="20" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="39" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="D20" s="39" t="s">
+        <v>129</v>
+      </c>
+      <c r="E20" s="40" t="s">
         <v>103</v>
       </c>
-      <c r="D8" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="38" t="s">
-        <v>104</v>
-      </c>
-      <c r="F8" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="39" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="37" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="C9" s="37" t="s">
-        <v>105</v>
-      </c>
-      <c r="D9" s="37" t="s">
-        <v>9</v>
-      </c>
-      <c r="E9" s="38" t="s">
-        <v>106</v>
-      </c>
-      <c r="F9" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="39" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="37" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="C10" s="37" t="s">
-        <v>107</v>
-      </c>
-      <c r="D10" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="E10" s="38" t="s">
-        <v>109</v>
-      </c>
-      <c r="F10" s="37"/>
-      <c r="G10" s="39"/>
-    </row>
-    <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="37" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="C11" s="37" t="s">
-        <v>110</v>
-      </c>
-      <c r="D11" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="E11" s="38" t="s">
-        <v>111</v>
-      </c>
-      <c r="F11" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="39" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="37" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="C12" s="37" t="s">
-        <v>112</v>
-      </c>
-      <c r="D12" s="37" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" s="38" t="s">
-        <v>113</v>
-      </c>
-      <c r="F12" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" s="39" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="37" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="C13" s="37" t="s">
-        <v>114</v>
-      </c>
-      <c r="D13" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="38" t="s">
-        <v>115</v>
-      </c>
-      <c r="F13" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="G13" s="39" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="44" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="44" t="s">
-        <v>90</v>
-      </c>
-      <c r="C14" s="44" t="s">
-        <v>116</v>
-      </c>
-      <c r="D14" s="44" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="45" t="s">
-        <v>117</v>
-      </c>
-      <c r="F14" s="44"/>
-      <c r="G14" s="44"/>
-    </row>
-    <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="44" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="44" t="s">
-        <v>90</v>
-      </c>
-      <c r="C15" s="44" t="s">
-        <v>118</v>
-      </c>
-      <c r="D15" s="44" t="s">
-        <v>34</v>
-      </c>
-      <c r="E15" s="45" t="s">
-        <v>119</v>
-      </c>
-      <c r="F15" s="44"/>
-      <c r="G15" s="44"/>
-    </row>
-    <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="44" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="40" t="s">
-        <v>90</v>
-      </c>
-      <c r="C16" s="40" t="s">
-        <v>120</v>
-      </c>
-      <c r="D16" s="40" t="s">
-        <v>43</v>
-      </c>
-      <c r="E16" s="41" t="s">
-        <v>121</v>
-      </c>
-      <c r="F16" s="40"/>
-      <c r="G16" s="44"/>
-    </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="37" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="C17" s="37" t="s">
-        <v>122</v>
-      </c>
-      <c r="D17" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="38" t="s">
-        <v>123</v>
-      </c>
-      <c r="F17" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="G17" s="39" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="37" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="C18" s="37" t="s">
-        <v>124</v>
-      </c>
-      <c r="D18" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="38" t="s">
-        <v>125</v>
-      </c>
-      <c r="F18" s="37" t="s">
-        <v>11</v>
-      </c>
-      <c r="G18" s="39" t="n">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="37" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="C19" s="37" t="s">
-        <v>126</v>
-      </c>
-      <c r="D19" s="37" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="38" t="s">
-        <v>92</v>
-      </c>
-      <c r="F19" s="37"/>
-      <c r="G19" s="39"/>
-    </row>
-    <row r="20" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="37" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="C20" s="37" t="s">
-        <v>127</v>
-      </c>
-      <c r="D20" s="37" t="s">
-        <v>128</v>
-      </c>
-      <c r="E20" s="38" t="s">
-        <v>102</v>
-      </c>
-      <c r="F20" s="37"/>
-      <c r="G20" s="39"/>
-    </row>
-    <row r="21" s="18" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="22" s="18" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="23" s="18" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" s="18" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="25" s="18" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="41"/>
+    </row>
+    <row r="21" s="34" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="22" s="34" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="23" s="34" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" s="34" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" s="34" customFormat="true" ht="19.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" display="https://leetcode.com/problems/repeated-dna-sequences/"/>

</xml_diff>

<commit_message>
Done with day 21
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="168">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -2769,7 +2769,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="48" width="61.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="48" width="14.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="48" width="77.77"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="48" width="24.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="48" width="17.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="48" width="24.49"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="48" width="55.93"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="48" width="60.79"/>
   </cols>
@@ -2835,8 +2836,12 @@
       <c r="E2" s="54" t="s">
         <v>133</v>
       </c>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
+      <c r="F2" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="55" t="n">
+        <v>21</v>
+      </c>
       <c r="H2" s="55"/>
       <c r="I2" s="50"/>
       <c r="J2" s="50"/>

</xml_diff>

<commit_message>
Done with day 22 - Interval pattern
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="168">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -2918,8 +2918,12 @@
       <c r="E4" s="54" t="s">
         <v>137</v>
       </c>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
+      <c r="F4" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="55" t="n">
+        <v>22</v>
+      </c>
       <c r="H4" s="55"/>
       <c r="I4" s="50"/>
       <c r="J4" s="50"/>
@@ -2998,8 +3002,12 @@
       <c r="E6" s="54" t="s">
         <v>142</v>
       </c>
-      <c r="F6" s="55"/>
-      <c r="G6" s="55"/>
+      <c r="F6" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="55" t="n">
+        <v>22</v>
+      </c>
       <c r="H6" s="55"/>
       <c r="I6" s="50"/>
       <c r="J6" s="50"/>

</xml_diff>

<commit_message>
Done with day 23
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="168">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -2879,8 +2879,12 @@
       <c r="E3" s="54" t="s">
         <v>135</v>
       </c>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
+      <c r="F3" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="55" t="n">
+        <v>23</v>
+      </c>
       <c r="H3" s="55"/>
       <c r="I3" s="50"/>
       <c r="J3" s="50"/>

</xml_diff>

<commit_message>
Done with day 24
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="169">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -460,6 +460,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/remove-covered-intervals/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Practice Sorting 2D Array acc to first or last element</t>
   </si>
   <si>
     <t xml:space="preserve">1094. Car Pooling</t>
@@ -1989,7 +1992,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
@@ -2012,7 +2015,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
@@ -2035,7 +2038,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
@@ -2058,7 +2061,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
@@ -2081,7 +2084,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <v>5</v>
       </c>
@@ -2104,7 +2107,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
         <v>6</v>
       </c>
@@ -2127,7 +2130,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
         <v>7</v>
       </c>
@@ -2150,7 +2153,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>8</v>
       </c>
@@ -2173,7 +2176,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>9</v>
       </c>
@@ -2196,7 +2199,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>10</v>
       </c>
@@ -2219,7 +2222,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>11</v>
       </c>
@@ -3049,9 +3052,15 @@
       <c r="E7" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="F7" s="55"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="55"/>
+      <c r="F7" s="55" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="55" t="n">
+        <v>24</v>
+      </c>
+      <c r="H7" s="55" t="s">
+        <v>145</v>
+      </c>
       <c r="I7" s="50"/>
       <c r="J7" s="50"/>
       <c r="K7" s="50"/>
@@ -3080,13 +3089,13 @@
         <v>131</v>
       </c>
       <c r="C8" s="53" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D8" s="53" t="s">
         <v>19</v>
       </c>
       <c r="E8" s="54" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F8" s="55"/>
       <c r="G8" s="55"/>
@@ -3119,13 +3128,13 @@
         <v>131</v>
       </c>
       <c r="C9" s="53" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D9" s="53" t="s">
         <v>34</v>
       </c>
       <c r="E9" s="54" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F9" s="55"/>
       <c r="G9" s="55"/>
@@ -3158,13 +3167,13 @@
         <v>131</v>
       </c>
       <c r="C10" s="53" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D10" s="51" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="54" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F10" s="55"/>
       <c r="G10" s="55"/>
@@ -3197,7 +3206,7 @@
         <v>131</v>
       </c>
       <c r="C11" s="53" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D11" s="53" t="s">
         <v>19</v>
@@ -3236,7 +3245,7 @@
         <v>131</v>
       </c>
       <c r="C12" s="53" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D12" s="53" t="s">
         <v>19</v>
@@ -3275,7 +3284,7 @@
         <v>131</v>
       </c>
       <c r="C13" s="53" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D13" s="53" t="s">
         <v>19</v>
@@ -3314,7 +3323,7 @@
         <v>131</v>
       </c>
       <c r="C14" s="63" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D14" s="63" t="s">
         <v>19</v>
@@ -3351,7 +3360,7 @@
         <v>131</v>
       </c>
       <c r="C15" s="63" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D15" s="63" t="s">
         <v>19</v>
@@ -3388,13 +3397,13 @@
         <v>131</v>
       </c>
       <c r="C16" s="63" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D16" s="63" t="s">
         <v>19</v>
       </c>
       <c r="E16" s="64" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F16" s="65"/>
       <c r="G16" s="65"/>
@@ -3427,13 +3436,13 @@
         <v>131</v>
       </c>
       <c r="C17" s="53" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D17" s="51" t="s">
         <v>9</v>
       </c>
       <c r="E17" s="54" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F17" s="55"/>
       <c r="G17" s="55"/>
@@ -3466,13 +3475,13 @@
         <v>131</v>
       </c>
       <c r="C18" s="53" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D18" s="51" t="s">
         <v>19</v>
       </c>
       <c r="E18" s="54" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F18" s="55"/>
       <c r="G18" s="55"/>
@@ -3505,13 +3514,13 @@
         <v>131</v>
       </c>
       <c r="C19" s="53" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D19" s="51" t="s">
         <v>34</v>
       </c>
       <c r="E19" s="54" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F19" s="55"/>
       <c r="G19" s="55"/>
@@ -3544,13 +3553,13 @@
         <v>131</v>
       </c>
       <c r="C20" s="67" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D20" s="68" t="s">
         <v>19</v>
       </c>
       <c r="E20" s="69" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="F20" s="70"/>
       <c r="G20" s="70"/>
@@ -3583,13 +3592,13 @@
         <v>131</v>
       </c>
       <c r="C21" s="67" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D21" s="68" t="s">
         <v>19</v>
       </c>
       <c r="E21" s="69" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F21" s="70"/>
       <c r="G21" s="70"/>
@@ -3622,13 +3631,13 @@
         <v>131</v>
       </c>
       <c r="C22" s="67" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D22" s="68" t="s">
         <v>19</v>
       </c>
       <c r="E22" s="69" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F22" s="70"/>
       <c r="G22" s="70"/>
@@ -3661,13 +3670,13 @@
         <v>131</v>
       </c>
       <c r="C23" s="67" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D23" s="67" t="s">
         <v>34</v>
       </c>
       <c r="E23" s="69" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F23" s="70"/>
       <c r="G23" s="70"/>

</xml_diff>

<commit_message>
Done with day 27
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="171">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -3216,8 +3216,12 @@
       <c r="E11" s="53" t="s">
         <v>133</v>
       </c>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
+      <c r="F11" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="54" t="n">
+        <v>21</v>
+      </c>
       <c r="H11" s="54"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -3460,8 +3464,12 @@
       <c r="E17" s="53" t="s">
         <v>162</v>
       </c>
-      <c r="F17" s="54"/>
-      <c r="G17" s="54"/>
+      <c r="F17" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" s="54" t="n">
+        <v>27</v>
+      </c>
       <c r="H17" s="54"/>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -3499,8 +3507,12 @@
       <c r="E18" s="53" t="s">
         <v>164</v>
       </c>
-      <c r="F18" s="54"/>
-      <c r="G18" s="54"/>
+      <c r="F18" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" s="54" t="n">
+        <v>27</v>
+      </c>
       <c r="H18" s="54"/>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>

</xml_diff>

<commit_message>
Done with day 29 - Line Sweep Algo
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="174">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -486,6 +486,9 @@
     <t xml:space="preserve">https://www.geeksforgeeks.org/problems/attend-all-meetings-ii/1</t>
   </si>
   <si>
+    <t xml:space="preserve">Line Sweep Algo Practice</t>
+  </si>
+  <si>
     <t xml:space="preserve">56. Merge Intervals (Brute Force)</t>
   </si>
   <si>
@@ -522,34 +525,10 @@
     <t xml:space="preserve">https://www.geeksforgeeks.org/problems/attend-all-meetings/1</t>
   </si>
   <si>
-    <t xml:space="preserve">Line Sweep Algo Practice</t>
-  </si>
-  <si>
     <t xml:space="preserve">729. My Calendar I (Brute Force + Line Sweep)</t>
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/my-calendar-i/description/</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Comic Sans MS"/>
-        <family val="4"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Line Sweep Algo</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Comic Sans MS"/>
-        <family val="4"/>
-      </rPr>
-      <t xml:space="preserve"> Practice</t>
-    </r>
   </si>
   <si>
     <t xml:space="preserve">732. My Calendar III (Line Sweep)</t>
@@ -1110,10 +1089,6 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1131,6 +1106,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="21" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2034,7 +2013,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
@@ -2057,7 +2036,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
@@ -2080,7 +2059,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
@@ -2103,7 +2082,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
@@ -2126,7 +2105,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <v>5</v>
       </c>
@@ -2149,7 +2128,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
         <v>6</v>
       </c>
@@ -2172,7 +2151,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
         <v>7</v>
       </c>
@@ -2195,7 +2174,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>8</v>
       </c>
@@ -2218,7 +2197,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>9</v>
       </c>
@@ -2241,7 +2220,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>10</v>
       </c>
@@ -2264,7 +2243,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>11</v>
       </c>
@@ -3223,9 +3202,15 @@
       <c r="E10" s="53" t="s">
         <v>152</v>
       </c>
-      <c r="F10" s="54"/>
-      <c r="G10" s="54"/>
-      <c r="H10" s="54"/>
+      <c r="F10" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="54" t="n">
+        <v>29</v>
+      </c>
+      <c r="H10" s="54" t="s">
+        <v>153</v>
+      </c>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
       <c r="K10" s="2"/>
@@ -3254,7 +3239,7 @@
         <v>131</v>
       </c>
       <c r="C11" s="52" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D11" s="52" t="s">
         <v>19</v>
@@ -3297,7 +3282,7 @@
         <v>131</v>
       </c>
       <c r="C12" s="52" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D12" s="52" t="s">
         <v>19</v>
@@ -3336,7 +3321,7 @@
         <v>131</v>
       </c>
       <c r="C13" s="52" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D13" s="52" t="s">
         <v>19</v>
@@ -3375,7 +3360,7 @@
         <v>131</v>
       </c>
       <c r="C14" s="62" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D14" s="62" t="s">
         <v>19</v>
@@ -3387,8 +3372,8 @@
       <c r="G14" s="64" t="n">
         <v>25</v>
       </c>
-      <c r="H14" s="65" t="s">
-        <v>157</v>
+      <c r="H14" s="64" t="s">
+        <v>158</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -3418,7 +3403,7 @@
         <v>131</v>
       </c>
       <c r="C15" s="62" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D15" s="62" t="s">
         <v>19</v>
@@ -3430,8 +3415,8 @@
       <c r="G15" s="64" t="n">
         <v>25</v>
       </c>
-      <c r="H15" s="65" t="s">
-        <v>157</v>
+      <c r="H15" s="64" t="s">
+        <v>158</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -3461,22 +3446,22 @@
         <v>131</v>
       </c>
       <c r="C16" s="62" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D16" s="62" t="s">
         <v>19</v>
       </c>
       <c r="E16" s="63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F16" s="64" t="s">
         <v>11</v>
       </c>
       <c r="G16" s="64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H16" s="64" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -3506,13 +3491,13 @@
         <v>131</v>
       </c>
       <c r="C17" s="52" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D17" s="50" t="s">
         <v>9</v>
       </c>
       <c r="E17" s="53" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="F17" s="54" t="s">
         <v>11</v>
@@ -3521,7 +3506,7 @@
         <v>27</v>
       </c>
       <c r="H17" s="64" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
       <c r="I17" s="2"/>
       <c r="J17" s="2"/>
@@ -3566,7 +3551,7 @@
         <v>27</v>
       </c>
       <c r="H18" s="64" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2"/>
@@ -3596,18 +3581,22 @@
         <v>131</v>
       </c>
       <c r="C19" s="52" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D19" s="50" t="s">
         <v>34</v>
       </c>
       <c r="E19" s="53" t="s">
-        <v>170</v>
-      </c>
-      <c r="F19" s="54"/>
-      <c r="G19" s="54"/>
+        <v>169</v>
+      </c>
+      <c r="F19" s="54" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" s="54" t="n">
+        <v>29</v>
+      </c>
       <c r="H19" s="64" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
@@ -3633,25 +3622,27 @@
       <c r="A20" s="38" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="66" t="s">
+      <c r="B20" s="65" t="s">
         <v>131</v>
       </c>
-      <c r="C20" s="67" t="s">
-        <v>171</v>
-      </c>
-      <c r="D20" s="68" t="s">
+      <c r="C20" s="66" t="s">
+        <v>170</v>
+      </c>
+      <c r="D20" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="69" t="s">
+      <c r="E20" s="68" t="s">
         <v>167</v>
       </c>
-      <c r="F20" s="70" t="s">
+      <c r="F20" s="69" t="s">
         <v>11</v>
       </c>
-      <c r="G20" s="70" t="n">
+      <c r="G20" s="69" t="n">
         <v>27</v>
       </c>
-      <c r="H20" s="70"/>
+      <c r="H20" s="70" t="s">
+        <v>153</v>
+      </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
@@ -3673,24 +3664,24 @@
       <c r="AA20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="68" t="n">
+      <c r="A21" s="67" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="66" t="s">
+      <c r="B21" s="65" t="s">
         <v>131</v>
       </c>
-      <c r="C21" s="67" t="s">
-        <v>172</v>
-      </c>
-      <c r="D21" s="68" t="s">
+      <c r="C21" s="66" t="s">
+        <v>171</v>
+      </c>
+      <c r="D21" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="69" t="s">
+      <c r="E21" s="68" t="s">
         <v>152</v>
       </c>
-      <c r="F21" s="70"/>
-      <c r="G21" s="70"/>
-      <c r="H21" s="70"/>
+      <c r="F21" s="69"/>
+      <c r="G21" s="69"/>
+      <c r="H21" s="69"/>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
@@ -3712,24 +3703,24 @@
       <c r="AA21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="68" t="n">
+      <c r="A22" s="67" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="66" t="s">
+      <c r="B22" s="65" t="s">
         <v>131</v>
       </c>
-      <c r="C22" s="67" t="s">
-        <v>173</v>
-      </c>
-      <c r="D22" s="68" t="s">
+      <c r="C22" s="66" t="s">
+        <v>172</v>
+      </c>
+      <c r="D22" s="67" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="69" t="s">
+      <c r="E22" s="68" t="s">
         <v>152</v>
       </c>
-      <c r="F22" s="70"/>
-      <c r="G22" s="70"/>
-      <c r="H22" s="70"/>
+      <c r="F22" s="69"/>
+      <c r="G22" s="69"/>
+      <c r="H22" s="69"/>
       <c r="I22" s="2"/>
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
@@ -3751,24 +3742,24 @@
       <c r="AA22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="68" t="n">
+      <c r="A23" s="67" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="66" t="s">
+      <c r="B23" s="65" t="s">
         <v>131</v>
       </c>
-      <c r="C23" s="67" t="s">
-        <v>174</v>
-      </c>
-      <c r="D23" s="67" t="s">
+      <c r="C23" s="66" t="s">
+        <v>173</v>
+      </c>
+      <c r="D23" s="66" t="s">
         <v>34</v>
       </c>
-      <c r="E23" s="69" t="s">
+      <c r="E23" s="68" t="s">
         <v>150</v>
       </c>
-      <c r="F23" s="70"/>
-      <c r="G23" s="70"/>
-      <c r="H23" s="70"/>
+      <c r="F23" s="69"/>
+      <c r="G23" s="69"/>
+      <c r="H23" s="69"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>

</xml_diff>

<commit_message>
Done with day 32
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="206">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -599,6 +599,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/remove-duplicates-from-sorted-list/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Needs Practice</t>
   </si>
   <si>
     <t xml:space="preserve">203. Remove Linked List Elements</t>
@@ -2145,7 +2148,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
@@ -2168,7 +2171,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
@@ -2191,7 +2194,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
@@ -2214,7 +2217,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
@@ -2237,7 +2240,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <v>5</v>
       </c>
@@ -2260,7 +2263,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
         <v>6</v>
       </c>
@@ -2283,7 +2286,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
         <v>7</v>
       </c>
@@ -2306,7 +2309,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>8</v>
       </c>
@@ -2329,7 +2332,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>9</v>
       </c>
@@ -2352,7 +2355,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>10</v>
       </c>
@@ -2375,7 +2378,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>11</v>
       </c>
@@ -18203,9 +18206,15 @@
       <c r="E8" s="74" t="s">
         <v>190</v>
       </c>
-      <c r="F8" s="75"/>
-      <c r="G8" s="62"/>
-      <c r="H8" s="62"/>
+      <c r="F8" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" s="62" t="n">
+        <v>32</v>
+      </c>
+      <c r="H8" s="62" t="s">
+        <v>191</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="73" t="n">
@@ -18215,13 +18224,13 @@
         <v>175</v>
       </c>
       <c r="C9" s="73" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D9" s="73" t="s">
         <v>9</v>
       </c>
       <c r="E9" s="74" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F9" s="75" t="s">
         <v>11</v>
@@ -18230,7 +18239,7 @@
         <v>32</v>
       </c>
       <c r="H9" s="62" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18241,13 +18250,13 @@
         <v>175</v>
       </c>
       <c r="C10" s="73" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D10" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="74" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F10" s="75"/>
       <c r="G10" s="62"/>
@@ -18261,13 +18270,13 @@
         <v>175</v>
       </c>
       <c r="C11" s="73" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D11" s="73" t="s">
         <v>43</v>
       </c>
       <c r="E11" s="74" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="F11" s="75"/>
       <c r="G11" s="62"/>
@@ -18281,13 +18290,13 @@
         <v>175</v>
       </c>
       <c r="C12" s="73" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D12" s="73" t="s">
         <v>43</v>
       </c>
       <c r="E12" s="74" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F12" s="75"/>
       <c r="G12" s="62"/>
@@ -18301,13 +18310,13 @@
         <v>175</v>
       </c>
       <c r="C13" s="73" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D13" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E13" s="74" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F13" s="75"/>
       <c r="G13" s="62"/>
@@ -18321,13 +18330,13 @@
         <v>175</v>
       </c>
       <c r="C14" s="73" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D14" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="74" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F14" s="75"/>
       <c r="G14" s="62"/>
@@ -18341,7 +18350,7 @@
         <v>175</v>
       </c>
       <c r="C15" s="73" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D15" s="73" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Done with day 33
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="207">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -575,6 +575,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/reverse-linked-list-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Popular Interview Que</t>
   </si>
   <si>
     <t xml:space="preserve">143. Reorder List</t>
@@ -2148,7 +2151,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
@@ -2171,7 +2174,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
@@ -2194,7 +2197,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
@@ -2217,7 +2220,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
@@ -2240,7 +2243,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <v>5</v>
       </c>
@@ -2263,7 +2266,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
         <v>6</v>
       </c>
@@ -2286,7 +2289,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
         <v>7</v>
       </c>
@@ -2309,7 +2312,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>8</v>
       </c>
@@ -2332,7 +2335,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>9</v>
       </c>
@@ -2355,7 +2358,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>10</v>
       </c>
@@ -2378,7 +2381,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>11</v>
       </c>
@@ -18126,9 +18129,15 @@
       <c r="E4" s="74" t="s">
         <v>182</v>
       </c>
-      <c r="F4" s="75"/>
-      <c r="G4" s="62"/>
-      <c r="H4" s="62"/>
+      <c r="F4" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="62" t="n">
+        <v>33</v>
+      </c>
+      <c r="H4" s="62" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="73" t="n">
@@ -18138,17 +18147,23 @@
         <v>175</v>
       </c>
       <c r="C5" s="73" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D5" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E5" s="74" t="s">
-        <v>184</v>
-      </c>
-      <c r="F5" s="75"/>
-      <c r="G5" s="62"/>
-      <c r="H5" s="62"/>
+        <v>185</v>
+      </c>
+      <c r="F5" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" s="62" t="n">
+        <v>33</v>
+      </c>
+      <c r="H5" s="62" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="73" t="n">
@@ -18158,13 +18173,13 @@
         <v>175</v>
       </c>
       <c r="C6" s="73" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D6" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="74" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F6" s="75"/>
       <c r="G6" s="62"/>
@@ -18178,13 +18193,13 @@
         <v>175</v>
       </c>
       <c r="C7" s="73" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D7" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="74" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F7" s="75"/>
       <c r="G7" s="62"/>
@@ -18198,13 +18213,13 @@
         <v>175</v>
       </c>
       <c r="C8" s="73" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D8" s="73" t="s">
         <v>9</v>
       </c>
       <c r="E8" s="74" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F8" s="75" t="s">
         <v>11</v>
@@ -18213,7 +18228,7 @@
         <v>32</v>
       </c>
       <c r="H8" s="62" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18224,13 +18239,13 @@
         <v>175</v>
       </c>
       <c r="C9" s="73" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D9" s="73" t="s">
         <v>9</v>
       </c>
       <c r="E9" s="74" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F9" s="75" t="s">
         <v>11</v>
@@ -18239,7 +18254,7 @@
         <v>32</v>
       </c>
       <c r="H9" s="62" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18250,13 +18265,13 @@
         <v>175</v>
       </c>
       <c r="C10" s="73" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D10" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="74" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F10" s="75"/>
       <c r="G10" s="62"/>
@@ -18270,13 +18285,13 @@
         <v>175</v>
       </c>
       <c r="C11" s="73" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D11" s="73" t="s">
         <v>43</v>
       </c>
       <c r="E11" s="74" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F11" s="75"/>
       <c r="G11" s="62"/>
@@ -18290,13 +18305,13 @@
         <v>175</v>
       </c>
       <c r="C12" s="73" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D12" s="73" t="s">
         <v>43</v>
       </c>
       <c r="E12" s="74" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F12" s="75"/>
       <c r="G12" s="62"/>
@@ -18310,13 +18325,13 @@
         <v>175</v>
       </c>
       <c r="C13" s="73" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D13" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E13" s="74" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F13" s="75"/>
       <c r="G13" s="62"/>
@@ -18330,13 +18345,13 @@
         <v>175</v>
       </c>
       <c r="C14" s="73" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D14" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="74" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F14" s="75"/>
       <c r="G14" s="62"/>
@@ -18350,7 +18365,7 @@
         <v>175</v>
       </c>
       <c r="C15" s="73" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D15" s="73" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Done with day 34
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="210">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -577,7 +577,7 @@
     <t xml:space="preserve">https://leetcode.com/problems/reverse-linked-list-ii/</t>
   </si>
   <si>
-    <t xml:space="preserve">Popular Interview Que</t>
+    <t xml:space="preserve">Popular Interview Que (Imp)</t>
   </si>
   <si>
     <t xml:space="preserve">143. Reorder List</t>
@@ -586,12 +586,18 @@
     <t xml:space="preserve">https://leetcode.com/problems/reorder-list/</t>
   </si>
   <si>
+    <t xml:space="preserve">Popular Interview Que ( Merging two LL –Math Trick )</t>
+  </si>
+  <si>
     <t xml:space="preserve">1721. Swapping Nodes in a Linked List</t>
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/swapping-nodes-in-a-linked-list/</t>
   </si>
   <si>
+    <t xml:space="preserve">How to reach same distance from start and end</t>
+  </si>
+  <si>
     <t xml:space="preserve">2074. Reverse Nodes in Even Length Groups</t>
   </si>
   <si>
@@ -638,6 +644,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/odd-even-linked-list/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Popular Interview Que (classic prob. of rearrangement of nodes)</t>
   </si>
   <si>
     <t xml:space="preserve">24. Swap Nodes in Pairs</t>
@@ -2151,7 +2160,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
@@ -2174,7 +2183,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
@@ -2197,7 +2206,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
@@ -2220,7 +2229,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
@@ -2243,7 +2252,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <v>5</v>
       </c>
@@ -2266,7 +2275,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
         <v>6</v>
       </c>
@@ -2289,7 +2298,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
         <v>7</v>
       </c>
@@ -2312,7 +2321,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>8</v>
       </c>
@@ -2335,7 +2344,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>9</v>
       </c>
@@ -2358,7 +2367,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>10</v>
       </c>
@@ -2381,7 +2390,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>11</v>
       </c>
@@ -18032,12 +18041,12 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="69" width="6.96"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="69" width="42.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="69" width="62.42"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="4" min="4" style="69" width="11.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="69" width="94.89"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="69" width="11.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="69" width="10.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="69" width="47.12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="69" width="57.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="69" width="14.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="69" width="107.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="69" width="9.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="69" width="8.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="69" width="79.21"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="69" width="11.55"/>
   </cols>
   <sheetData>
@@ -18162,7 +18171,7 @@
         <v>33</v>
       </c>
       <c r="H5" s="62" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18173,17 +18182,23 @@
         <v>175</v>
       </c>
       <c r="C6" s="73" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D6" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E6" s="74" t="s">
-        <v>187</v>
-      </c>
-      <c r="F6" s="75"/>
-      <c r="G6" s="62"/>
-      <c r="H6" s="62"/>
+        <v>188</v>
+      </c>
+      <c r="F6" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="62" t="n">
+        <v>34</v>
+      </c>
+      <c r="H6" s="62" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="73" t="n">
@@ -18193,13 +18208,13 @@
         <v>175</v>
       </c>
       <c r="C7" s="73" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D7" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E7" s="74" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F7" s="75"/>
       <c r="G7" s="62"/>
@@ -18213,13 +18228,13 @@
         <v>175</v>
       </c>
       <c r="C8" s="73" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D8" s="73" t="s">
         <v>9</v>
       </c>
       <c r="E8" s="74" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F8" s="75" t="s">
         <v>11</v>
@@ -18228,7 +18243,7 @@
         <v>32</v>
       </c>
       <c r="H8" s="62" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18239,13 +18254,13 @@
         <v>175</v>
       </c>
       <c r="C9" s="73" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D9" s="73" t="s">
         <v>9</v>
       </c>
       <c r="E9" s="74" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F9" s="75" t="s">
         <v>11</v>
@@ -18254,7 +18269,7 @@
         <v>32</v>
       </c>
       <c r="H9" s="62" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18265,13 +18280,13 @@
         <v>175</v>
       </c>
       <c r="C10" s="73" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D10" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="74" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F10" s="75"/>
       <c r="G10" s="62"/>
@@ -18285,13 +18300,13 @@
         <v>175</v>
       </c>
       <c r="C11" s="73" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D11" s="73" t="s">
         <v>43</v>
       </c>
       <c r="E11" s="74" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F11" s="75"/>
       <c r="G11" s="62"/>
@@ -18305,13 +18320,13 @@
         <v>175</v>
       </c>
       <c r="C12" s="73" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D12" s="73" t="s">
         <v>43</v>
       </c>
       <c r="E12" s="74" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F12" s="75"/>
       <c r="G12" s="62"/>
@@ -18325,17 +18340,23 @@
         <v>175</v>
       </c>
       <c r="C13" s="73" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D13" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E13" s="74" t="s">
-        <v>203</v>
-      </c>
-      <c r="F13" s="75"/>
-      <c r="G13" s="62"/>
-      <c r="H13" s="62"/>
+        <v>205</v>
+      </c>
+      <c r="F13" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="62" t="n">
+        <v>34</v>
+      </c>
+      <c r="H13" s="62" t="s">
+        <v>206</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="73" t="n">
@@ -18345,13 +18366,13 @@
         <v>175</v>
       </c>
       <c r="C14" s="73" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D14" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="74" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F14" s="75"/>
       <c r="G14" s="62"/>
@@ -18365,7 +18386,7 @@
         <v>175</v>
       </c>
       <c r="C15" s="73" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D15" s="73" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Done with day 35
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="211">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -626,6 +626,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/split-linked-list-in-parts/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design Linked List pattern</t>
   </si>
   <si>
     <t xml:space="preserve">Delete N Nodes After M Nodes of a Linked List</t>
@@ -18288,9 +18291,15 @@
       <c r="E10" s="74" t="s">
         <v>199</v>
       </c>
-      <c r="F10" s="75"/>
-      <c r="G10" s="62"/>
-      <c r="H10" s="62"/>
+      <c r="F10" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" s="62" t="n">
+        <v>35</v>
+      </c>
+      <c r="H10" s="62" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="73" t="n">
@@ -18300,13 +18309,13 @@
         <v>175</v>
       </c>
       <c r="C11" s="73" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D11" s="73" t="s">
         <v>43</v>
       </c>
       <c r="E11" s="74" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F11" s="75"/>
       <c r="G11" s="62"/>
@@ -18320,13 +18329,13 @@
         <v>175</v>
       </c>
       <c r="C12" s="73" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D12" s="73" t="s">
         <v>43</v>
       </c>
       <c r="E12" s="74" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F12" s="75"/>
       <c r="G12" s="62"/>
@@ -18340,13 +18349,13 @@
         <v>175</v>
       </c>
       <c r="C13" s="73" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D13" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E13" s="74" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F13" s="75" t="s">
         <v>11</v>
@@ -18355,7 +18364,7 @@
         <v>34</v>
       </c>
       <c r="H13" s="62" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18366,16 +18375,20 @@
         <v>175</v>
       </c>
       <c r="C14" s="73" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D14" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="74" t="s">
-        <v>208</v>
-      </c>
-      <c r="F14" s="75"/>
-      <c r="G14" s="62"/>
+        <v>209</v>
+      </c>
+      <c r="F14" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="62" t="n">
+        <v>35</v>
+      </c>
       <c r="H14" s="62"/>
     </row>
     <row r="15" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18386,7 +18399,7 @@
         <v>175</v>
       </c>
       <c r="C15" s="73" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D15" s="73" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Done with day 36
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="211">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -18121,8 +18121,12 @@
       <c r="E3" s="74" t="s">
         <v>180</v>
       </c>
-      <c r="F3" s="75"/>
-      <c r="G3" s="62"/>
+      <c r="F3" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" s="62" t="n">
+        <v>36</v>
+      </c>
       <c r="H3" s="62"/>
     </row>
     <row r="4" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Done with day 37
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="213">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -604,6 +604,9 @@
     <t xml:space="preserve">https://leetcode.com/problems/reverse-nodes-in-even-length-groups/</t>
   </si>
   <si>
+    <t xml:space="preserve">Must solve Interview Problem (Tests all the concepts learned so far)</t>
+  </si>
+  <si>
     <t xml:space="preserve">83. Remove Duplicates from Sorted List</t>
   </si>
   <si>
@@ -635,6 +638,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/delete-n-nodes-after-m-nodes-of-a-linked-list/description/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GFG</t>
   </si>
   <si>
     <t xml:space="preserve">Insert into a Sorted Circular Linked List</t>
@@ -2163,7 +2169,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="22" t="n">
         <v>1</v>
       </c>
@@ -2186,7 +2192,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="22" t="n">
         <v>2</v>
       </c>
@@ -2209,7 +2215,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="22" t="n">
         <v>3</v>
       </c>
@@ -2232,7 +2238,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
@@ -2255,7 +2261,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="22" t="n">
         <v>5</v>
       </c>
@@ -2278,7 +2284,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="n">
         <v>6</v>
       </c>
@@ -2301,7 +2307,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="n">
         <v>7</v>
       </c>
@@ -2324,7 +2330,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="30" t="n">
         <v>8</v>
       </c>
@@ -2347,7 +2353,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="22" t="n">
         <v>9</v>
       </c>
@@ -2370,7 +2376,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="n">
         <v>10</v>
       </c>
@@ -2393,7 +2399,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="22" t="n">
         <v>11</v>
       </c>
@@ -18223,9 +18229,15 @@
       <c r="E7" s="74" t="s">
         <v>191</v>
       </c>
-      <c r="F7" s="75"/>
-      <c r="G7" s="62"/>
-      <c r="H7" s="62"/>
+      <c r="F7" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="62" t="n">
+        <v>37</v>
+      </c>
+      <c r="H7" s="62" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="73" t="n">
@@ -18235,13 +18247,13 @@
         <v>175</v>
       </c>
       <c r="C8" s="73" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D8" s="73" t="s">
         <v>9</v>
       </c>
       <c r="E8" s="74" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F8" s="75" t="s">
         <v>11</v>
@@ -18250,7 +18262,7 @@
         <v>32</v>
       </c>
       <c r="H8" s="62" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18261,13 +18273,13 @@
         <v>175</v>
       </c>
       <c r="C9" s="73" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="D9" s="73" t="s">
         <v>9</v>
       </c>
       <c r="E9" s="74" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F9" s="75" t="s">
         <v>11</v>
@@ -18276,7 +18288,7 @@
         <v>32</v>
       </c>
       <c r="H9" s="62" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18287,13 +18299,13 @@
         <v>175</v>
       </c>
       <c r="C10" s="73" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D10" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E10" s="74" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F10" s="75" t="s">
         <v>11</v>
@@ -18302,7 +18314,7 @@
         <v>35</v>
       </c>
       <c r="H10" s="62" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18313,17 +18325,23 @@
         <v>175</v>
       </c>
       <c r="C11" s="73" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D11" s="73" t="s">
         <v>43</v>
       </c>
       <c r="E11" s="74" t="s">
-        <v>202</v>
-      </c>
-      <c r="F11" s="75"/>
-      <c r="G11" s="62"/>
-      <c r="H11" s="62"/>
+        <v>203</v>
+      </c>
+      <c r="F11" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="62" t="n">
+        <v>37</v>
+      </c>
+      <c r="H11" s="62" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="73" t="n">
@@ -18333,13 +18351,13 @@
         <v>175</v>
       </c>
       <c r="C12" s="73" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D12" s="73" t="s">
         <v>43</v>
       </c>
       <c r="E12" s="74" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F12" s="75"/>
       <c r="G12" s="62"/>
@@ -18353,13 +18371,13 @@
         <v>175</v>
       </c>
       <c r="C13" s="73" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D13" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E13" s="74" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F13" s="75" t="s">
         <v>11</v>
@@ -18368,7 +18386,7 @@
         <v>34</v>
       </c>
       <c r="H13" s="62" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18379,13 +18397,13 @@
         <v>175</v>
       </c>
       <c r="C14" s="73" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D14" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="74" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F14" s="75" t="s">
         <v>11</v>
@@ -18403,14 +18421,18 @@
         <v>175</v>
       </c>
       <c r="C15" s="73" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D15" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E15" s="75"/>
-      <c r="F15" s="75"/>
-      <c r="G15" s="62"/>
+      <c r="F15" s="75" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" s="62" t="n">
+        <v>32</v>
+      </c>
       <c r="H15" s="62"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Done with day 38
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="214">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -647,6 +647,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://neetcode.io/problems/insert-into-a-sorted-circular-linked-list/question</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neetcode</t>
   </si>
   <si>
     <t xml:space="preserve">328. Odd Even Linked List</t>
@@ -18360,8 +18363,12 @@
         <v>206</v>
       </c>
       <c r="F12" s="75"/>
-      <c r="G12" s="62"/>
-      <c r="H12" s="62"/>
+      <c r="G12" s="62" t="n">
+        <v>38</v>
+      </c>
+      <c r="H12" s="62" t="s">
+        <v>207</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="73" t="n">
@@ -18371,13 +18378,13 @@
         <v>175</v>
       </c>
       <c r="C13" s="73" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D13" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E13" s="74" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F13" s="75" t="s">
         <v>11</v>
@@ -18386,7 +18393,7 @@
         <v>34</v>
       </c>
       <c r="H13" s="62" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18397,13 +18404,13 @@
         <v>175</v>
       </c>
       <c r="C14" s="73" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D14" s="73" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="74" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F14" s="75" t="s">
         <v>11</v>
@@ -18421,7 +18428,7 @@
         <v>175</v>
       </c>
       <c r="C15" s="73" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D15" s="73" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Solve Pascal's Triangle II
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="506" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="220">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -55,6 +55,12 @@
   </si>
   <si>
     <t xml:space="preserve">https://youtu.be/ELo7RR-Isjk?si=4BAHl-pa8-hBILgE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pascal’s Triangle II</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/pascals-triangle-ii/</t>
   </si>
   <si>
     <t xml:space="preserve">Pattern</t>
@@ -984,12 +990,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="75">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1269,10 +1275,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="20" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1538,7 +1540,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="16.15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.78"/>
@@ -1550,7 +1552,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="11.53"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1585,12 +1587,27 @@
       </c>
       <c r="E2" s="1" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>119</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" display="https://leetcode.com/problems/pascals-triangle/"/>
     <hyperlink ref="E2" r:id="rId2" display="https://youtu.be/ELo7RR-Isjk?si=4BAHl-pa8-hBILgE"/>
+    <hyperlink ref="D3" r:id="rId3" display="https://leetcode.com/problems/pascals-triangle-ii/"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -1625,7 +1642,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>1</v>
@@ -1637,10 +1654,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1648,19 +1665,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G2" s="8" t="n">
         <v>3</v>
@@ -1671,19 +1688,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" s="9" t="s">
         <v>18</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>16</v>
       </c>
       <c r="G3" s="8" t="n">
         <v>2</v>
@@ -1694,19 +1711,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G4" s="8" t="n">
         <v>3</v>
@@ -1717,19 +1734,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G5" s="8" t="n">
         <v>3</v>
@@ -1740,19 +1757,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>3</v>
@@ -1763,19 +1780,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C7" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="9" t="s">
-        <v>24</v>
-      </c>
       <c r="E7" s="10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G7" s="8" t="n">
         <v>3</v>
@@ -1786,19 +1803,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>4</v>
@@ -1809,19 +1826,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G9" s="8" t="n">
         <v>4</v>
@@ -1832,19 +1849,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>6</v>
@@ -1855,19 +1872,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>6</v>
@@ -1878,19 +1895,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>6</v>
@@ -1901,16 +1918,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F13" s="12"/>
       <c r="G13" s="14"/>
@@ -1920,16 +1937,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C14" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="12" t="s">
-        <v>39</v>
-      </c>
       <c r="E14" s="13" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="14"/>
@@ -1939,16 +1956,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C15" s="12" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D15" s="12" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F15" s="12"/>
       <c r="G15" s="14"/>
@@ -1958,16 +1975,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F16" s="12"/>
       <c r="G16" s="14"/>
@@ -1977,19 +1994,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G17" s="17" t="n">
         <v>2</v>
@@ -2000,19 +2017,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>5</v>
@@ -2023,22 +2040,22 @@
         <v>18</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E19" s="19" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G19" s="20" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2046,19 +2063,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G20" s="8" t="n">
         <v>5</v>
@@ -2069,22 +2086,22 @@
         <v>20</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E21" s="19" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G21" s="20" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2092,19 +2109,19 @@
         <v>21</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G22" s="8" t="n">
         <v>5</v>
@@ -2115,19 +2132,19 @@
         <v>22</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G23" s="8" t="n">
         <v>2</v>
@@ -2138,19 +2155,19 @@
         <v>23</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>2</v>
@@ -2161,19 +2178,19 @@
         <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G25" s="8" t="n">
         <v>2</v>
@@ -2184,19 +2201,19 @@
         <v>25</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>4</v>
@@ -2236,7 +2253,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C1" s="23" t="s">
         <v>1</v>
@@ -2248,260 +2265,260 @@
         <v>3</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G1" s="24" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="25" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D2" s="26" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="27" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F2" s="26" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G2" s="28" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="25" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D3" s="26" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="27" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G3" s="28" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="25" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D4" s="26" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="27" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F4" s="26" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G4" s="28" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="29" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F5" s="30" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G5" s="32" t="n">
         <v>11</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="25" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="25" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D7" s="26" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="27" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="25" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E8" s="27" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G8" s="28" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="33" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F9" s="34" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G9" s="36" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="25" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E10" s="27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G10" s="28" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="25" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F11" s="26" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G11" s="28" t="n">
         <v>8</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="25" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E12" s="27" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F12" s="26" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G12" s="28" t="n">
         <v>9</v>
@@ -2566,7 +2583,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="39" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C1" s="39" t="s">
         <v>1</v>
@@ -2578,10 +2595,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="39" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G1" s="40" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="27.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2589,19 +2606,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C2" s="42" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D2" s="42" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E2" s="43" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F2" s="42" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G2" s="44" t="n">
         <v>15</v>
@@ -2612,16 +2629,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D3" s="45" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E3" s="46" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F3" s="45"/>
       <c r="G3" s="45"/>
@@ -2631,16 +2648,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="47" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C4" s="47" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D4" s="47" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E4" s="48" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F4" s="47"/>
       <c r="G4" s="47"/>
@@ -2650,19 +2667,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E5" s="43" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F5" s="42" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="G5" s="44" t="n">
         <v>18</v>
@@ -2673,16 +2690,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="49" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C6" s="49" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D6" s="49" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E6" s="50" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F6" s="49"/>
       <c r="G6" s="49"/>
@@ -2692,19 +2709,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C7" s="42" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E7" s="43" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F7" s="42" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G7" s="44" t="n">
         <v>14</v>
@@ -2715,19 +2732,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C8" s="42" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E8" s="43" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F8" s="42" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G8" s="44" t="n">
         <v>13</v>
@@ -2738,19 +2755,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C9" s="42" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D9" s="42" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="43" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F9" s="42" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G9" s="44" t="n">
         <v>14</v>
@@ -2761,16 +2778,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C10" s="42" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E10" s="43" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F10" s="42"/>
       <c r="G10" s="44"/>
@@ -2780,19 +2797,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C11" s="42" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E11" s="43" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F11" s="42" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G11" s="44" t="n">
         <v>16</v>
@@ -2803,19 +2820,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C12" s="42" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D12" s="42" t="s">
         <v>7</v>
       </c>
       <c r="E12" s="43" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F12" s="42" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G12" s="44" t="n">
         <v>14</v>
@@ -2826,19 +2843,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C13" s="42" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E13" s="43" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F13" s="42" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G13" s="44" t="n">
         <v>17</v>
@@ -2849,16 +2866,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="49" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C14" s="49" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D14" s="49" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E14" s="50" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F14" s="49"/>
       <c r="G14" s="49"/>
@@ -2868,16 +2885,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C15" s="49" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D15" s="49" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E15" s="50" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F15" s="49"/>
       <c r="G15" s="49"/>
@@ -2887,16 +2904,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C16" s="45" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D16" s="45" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E16" s="46" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F16" s="45"/>
       <c r="G16" s="49"/>
@@ -2906,19 +2923,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C17" s="42" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E17" s="43" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F17" s="42" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G17" s="44" t="n">
         <v>13</v>
@@ -2929,19 +2946,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C18" s="42" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E18" s="43" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="F18" s="42" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G18" s="44" t="n">
         <v>13</v>
@@ -2952,16 +2969,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C19" s="42" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E19" s="43" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F19" s="42"/>
       <c r="G19" s="44"/>
@@ -2971,16 +2988,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="42" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C20" s="42" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="E20" s="43" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F20" s="42"/>
       <c r="G20" s="44"/>
@@ -3045,7 +3062,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>1</v>
@@ -3057,10 +3074,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>5</v>
@@ -3090,19 +3107,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C2" s="54" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D2" s="54" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E2" s="55" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F2" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G2" s="54" t="n">
         <v>21</v>
@@ -3133,19 +3150,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C3" s="54" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D3" s="54" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E3" s="55" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F3" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G3" s="54" t="n">
         <v>23</v>
@@ -3176,19 +3193,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C4" s="54" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D4" s="54" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E4" s="55" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F4" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G4" s="54" t="n">
         <v>22</v>
@@ -3219,21 +3236,21 @@
         <v>4</v>
       </c>
       <c r="B5" s="57" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C5" s="58" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D5" s="56" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E5" s="59" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F5" s="58"/>
       <c r="G5" s="58"/>
       <c r="H5" s="58" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
@@ -3260,19 +3277,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C6" s="54" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D6" s="54" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E6" s="55" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F6" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G6" s="54" t="n">
         <v>22</v>
@@ -3303,25 +3320,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C7" s="54" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D7" s="54" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E7" s="55" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F7" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G7" s="54" t="n">
         <v>24</v>
       </c>
       <c r="H7" s="54" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
@@ -3348,25 +3365,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C8" s="54" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D8" s="54" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E8" s="55" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F8" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G8" s="54" t="n">
         <v>28</v>
       </c>
       <c r="H8" s="54" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
@@ -3393,25 +3410,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C9" s="54" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D9" s="54" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E9" s="55" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F9" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G9" s="54" t="n">
         <v>30</v>
       </c>
       <c r="H9" s="54" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
@@ -3438,25 +3455,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C10" s="54" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D10" s="52" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E10" s="55" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F10" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G10" s="54" t="n">
         <v>29</v>
       </c>
       <c r="H10" s="54" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
@@ -3483,19 +3500,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C11" s="54" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D11" s="54" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E11" s="55" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F11" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G11" s="54" t="n">
         <v>21</v>
@@ -3526,16 +3543,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C12" s="54" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D12" s="54" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E12" s="55" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -3565,16 +3582,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C13" s="54" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D13" s="54" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E13" s="55" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F13" s="54"/>
       <c r="G13" s="54"/>
@@ -3604,23 +3621,23 @@
         <v>13</v>
       </c>
       <c r="B14" s="61" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C14" s="62" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D14" s="62" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E14" s="63"/>
       <c r="F14" s="64" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G14" s="64" t="n">
         <v>25</v>
       </c>
       <c r="H14" s="64" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
@@ -3647,23 +3664,23 @@
         <v>14</v>
       </c>
       <c r="B15" s="61" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C15" s="62" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D15" s="62" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E15" s="63"/>
       <c r="F15" s="64" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G15" s="64" t="n">
         <v>25</v>
       </c>
       <c r="H15" s="64" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
@@ -3690,25 +3707,25 @@
         <v>15</v>
       </c>
       <c r="B16" s="61" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C16" s="62" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D16" s="62" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E16" s="63" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F16" s="64" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G16" s="64" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="H16" s="64" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
@@ -3735,25 +3752,25 @@
         <v>16</v>
       </c>
       <c r="B17" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C17" s="54" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D17" s="52" t="s">
         <v>7</v>
       </c>
       <c r="E17" s="55" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F17" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G17" s="54" t="n">
         <v>27</v>
       </c>
       <c r="H17" s="64" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
@@ -3780,25 +3797,25 @@
         <v>17</v>
       </c>
       <c r="B18" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C18" s="54" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D18" s="52" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E18" s="55" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F18" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G18" s="54" t="n">
         <v>27</v>
       </c>
       <c r="H18" s="64" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
@@ -3825,25 +3842,25 @@
         <v>18</v>
       </c>
       <c r="B19" s="53" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C19" s="54" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D19" s="52" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E19" s="55" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F19" s="54" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G19" s="54" t="n">
         <v>29</v>
       </c>
       <c r="H19" s="64" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
@@ -3870,25 +3887,25 @@
         <v>19</v>
       </c>
       <c r="B20" s="66" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C20" s="67" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D20" s="68" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E20" s="69" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F20" s="67" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G20" s="67" t="n">
         <v>27</v>
       </c>
       <c r="H20" s="67" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
@@ -3915,16 +3932,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="66" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C21" s="67" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D21" s="68" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E21" s="69" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F21" s="67"/>
       <c r="G21" s="67"/>
@@ -3954,16 +3971,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="66" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C22" s="67" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D22" s="68" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E22" s="69" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F22" s="67"/>
       <c r="G22" s="67"/>
@@ -3993,16 +4010,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="66" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C23" s="67" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D23" s="67" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E23" s="69" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F23" s="67"/>
       <c r="G23" s="67"/>
@@ -18133,15 +18150,15 @@
   <dimension ref="A1:H15"/>
   <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="16.15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="71" width="6.96"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="71" width="42.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="71" width="57.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="71" width="14.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="71" width="107.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="71" width="9.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="71" width="8.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="71" width="79.21"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="71" width="11.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="57.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="107.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="79.21"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="1" width="11.55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18149,7 +18166,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -18161,59 +18178,59 @@
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="72" t="s">
-        <v>12</v>
-      </c>
-      <c r="H1" s="72" t="s">
+        <v>13</v>
+      </c>
+      <c r="G1" s="71" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="71" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="73" t="n">
+      <c r="A2" s="72" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C2" s="73" t="s">
-        <v>180</v>
-      </c>
-      <c r="D2" s="73" t="s">
+      <c r="B2" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C2" s="72" t="s">
+        <v>182</v>
+      </c>
+      <c r="D2" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="74" t="s">
-        <v>181</v>
-      </c>
-      <c r="F2" s="75" t="s">
-        <v>16</v>
+      <c r="E2" s="73" t="s">
+        <v>183</v>
+      </c>
+      <c r="F2" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G2" s="64" t="n">
         <v>32</v>
       </c>
       <c r="H2" s="64" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="73" t="n">
+      <c r="A3" s="72" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C3" s="73" t="s">
-        <v>183</v>
-      </c>
-      <c r="D3" s="73" t="s">
-        <v>39</v>
-      </c>
-      <c r="E3" s="74" t="s">
-        <v>184</v>
-      </c>
-      <c r="F3" s="75" t="s">
-        <v>16</v>
+      <c r="B3" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C3" s="72" t="s">
+        <v>185</v>
+      </c>
+      <c r="D3" s="72" t="s">
+        <v>41</v>
+      </c>
+      <c r="E3" s="73" t="s">
+        <v>186</v>
+      </c>
+      <c r="F3" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G3" s="64" t="n">
         <v>36</v>
@@ -18221,281 +18238,281 @@
       <c r="H3" s="64"/>
     </row>
     <row r="4" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="73" t="n">
+      <c r="A4" s="72" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C4" s="73" t="s">
-        <v>185</v>
-      </c>
-      <c r="D4" s="73" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="74" t="s">
-        <v>186</v>
-      </c>
-      <c r="F4" s="75" t="s">
-        <v>16</v>
+      <c r="B4" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C4" s="72" t="s">
+        <v>187</v>
+      </c>
+      <c r="D4" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="73" t="s">
+        <v>188</v>
+      </c>
+      <c r="F4" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G4" s="64" t="n">
         <v>33</v>
       </c>
       <c r="H4" s="64" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="73" t="n">
+      <c r="A5" s="72" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C5" s="73" t="s">
-        <v>188</v>
-      </c>
-      <c r="D5" s="73" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" s="74" t="s">
-        <v>189</v>
-      </c>
-      <c r="F5" s="75" t="s">
-        <v>16</v>
+      <c r="B5" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C5" s="72" t="s">
+        <v>190</v>
+      </c>
+      <c r="D5" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="73" t="s">
+        <v>191</v>
+      </c>
+      <c r="F5" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G5" s="64" t="n">
         <v>33</v>
       </c>
       <c r="H5" s="64" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="73" t="n">
+      <c r="A6" s="72" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C6" s="73" t="s">
-        <v>191</v>
-      </c>
-      <c r="D6" s="73" t="s">
-        <v>24</v>
-      </c>
-      <c r="E6" s="74" t="s">
-        <v>192</v>
-      </c>
-      <c r="F6" s="75" t="s">
-        <v>16</v>
+      <c r="B6" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C6" s="72" t="s">
+        <v>193</v>
+      </c>
+      <c r="D6" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="73" t="s">
+        <v>194</v>
+      </c>
+      <c r="F6" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G6" s="64" t="n">
         <v>34</v>
       </c>
       <c r="H6" s="64" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="73" t="n">
+      <c r="A7" s="72" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C7" s="73" t="s">
-        <v>194</v>
-      </c>
-      <c r="D7" s="73" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="74" t="s">
-        <v>195</v>
-      </c>
-      <c r="F7" s="75" t="s">
-        <v>16</v>
+      <c r="B7" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C7" s="72" t="s">
+        <v>196</v>
+      </c>
+      <c r="D7" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="73" t="s">
+        <v>197</v>
+      </c>
+      <c r="F7" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G7" s="64" t="n">
         <v>37</v>
       </c>
       <c r="H7" s="64" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="73" t="n">
+      <c r="A8" s="72" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C8" s="73" t="s">
-        <v>197</v>
-      </c>
-      <c r="D8" s="73" t="s">
+      <c r="B8" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C8" s="72" t="s">
+        <v>199</v>
+      </c>
+      <c r="D8" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="74" t="s">
-        <v>198</v>
-      </c>
-      <c r="F8" s="75" t="s">
-        <v>16</v>
+      <c r="E8" s="73" t="s">
+        <v>200</v>
+      </c>
+      <c r="F8" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G8" s="64" t="n">
         <v>32</v>
       </c>
       <c r="H8" s="64" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="73" t="n">
+      <c r="A9" s="72" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C9" s="73" t="s">
-        <v>200</v>
-      </c>
-      <c r="D9" s="73" t="s">
+      <c r="B9" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C9" s="72" t="s">
+        <v>202</v>
+      </c>
+      <c r="D9" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="74" t="s">
-        <v>201</v>
-      </c>
-      <c r="F9" s="75" t="s">
-        <v>16</v>
+      <c r="E9" s="73" t="s">
+        <v>203</v>
+      </c>
+      <c r="F9" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G9" s="64" t="n">
         <v>32</v>
       </c>
       <c r="H9" s="64" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="73" t="n">
+      <c r="A10" s="72" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C10" s="73" t="s">
-        <v>203</v>
-      </c>
-      <c r="D10" s="73" t="s">
-        <v>24</v>
-      </c>
-      <c r="E10" s="74" t="s">
-        <v>204</v>
-      </c>
-      <c r="F10" s="75" t="s">
-        <v>16</v>
+      <c r="B10" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C10" s="72" t="s">
+        <v>205</v>
+      </c>
+      <c r="D10" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="73" t="s">
+        <v>206</v>
+      </c>
+      <c r="F10" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G10" s="64" t="n">
         <v>35</v>
       </c>
       <c r="H10" s="64" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="73" t="n">
+      <c r="A11" s="72" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C11" s="73" t="s">
-        <v>206</v>
-      </c>
-      <c r="D11" s="73" t="s">
-        <v>48</v>
-      </c>
-      <c r="E11" s="74" t="s">
-        <v>207</v>
-      </c>
-      <c r="F11" s="75" t="s">
-        <v>16</v>
+      <c r="B11" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C11" s="72" t="s">
+        <v>208</v>
+      </c>
+      <c r="D11" s="72" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" s="73" t="s">
+        <v>209</v>
+      </c>
+      <c r="F11" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G11" s="64" t="n">
         <v>37</v>
       </c>
       <c r="H11" s="64" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="73" t="n">
+      <c r="A12" s="72" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C12" s="73" t="s">
-        <v>209</v>
-      </c>
-      <c r="D12" s="73" t="s">
-        <v>48</v>
-      </c>
-      <c r="E12" s="74" t="s">
-        <v>210</v>
-      </c>
-      <c r="F12" s="75"/>
+      <c r="B12" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C12" s="72" t="s">
+        <v>211</v>
+      </c>
+      <c r="D12" s="72" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" s="73" t="s">
+        <v>212</v>
+      </c>
+      <c r="F12" s="74"/>
       <c r="G12" s="64" t="n">
         <v>38</v>
       </c>
       <c r="H12" s="64" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="73" t="n">
+      <c r="A13" s="72" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C13" s="73" t="s">
-        <v>212</v>
-      </c>
-      <c r="D13" s="73" t="s">
-        <v>24</v>
-      </c>
-      <c r="E13" s="74" t="s">
-        <v>213</v>
-      </c>
-      <c r="F13" s="75" t="s">
-        <v>16</v>
+      <c r="B13" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C13" s="72" t="s">
+        <v>214</v>
+      </c>
+      <c r="D13" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="73" t="s">
+        <v>215</v>
+      </c>
+      <c r="F13" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G13" s="64" t="n">
         <v>34</v>
       </c>
       <c r="H13" s="64" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="73" t="n">
+      <c r="A14" s="72" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C14" s="73" t="s">
-        <v>215</v>
-      </c>
-      <c r="D14" s="73" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="74" t="s">
-        <v>216</v>
-      </c>
-      <c r="F14" s="75" t="s">
-        <v>16</v>
+      <c r="B14" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C14" s="72" t="s">
+        <v>217</v>
+      </c>
+      <c r="D14" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="E14" s="73" t="s">
+        <v>218</v>
+      </c>
+      <c r="F14" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G14" s="64" t="n">
         <v>35</v>
@@ -18503,21 +18520,21 @@
       <c r="H14" s="64"/>
     </row>
     <row r="15" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="73" t="n">
+      <c r="A15" s="72" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="73" t="s">
-        <v>179</v>
-      </c>
-      <c r="C15" s="73" t="s">
-        <v>217</v>
-      </c>
-      <c r="D15" s="73" t="s">
-        <v>24</v>
-      </c>
-      <c r="E15" s="75"/>
-      <c r="F15" s="75" t="s">
-        <v>16</v>
+      <c r="B15" s="72" t="s">
+        <v>181</v>
+      </c>
+      <c r="C15" s="72" t="s">
+        <v>219</v>
+      </c>
+      <c r="D15" s="72" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" s="74"/>
+      <c r="F15" s="74" t="s">
+        <v>18</v>
       </c>
       <c r="G15" s="64" t="n">
         <v>32</v>

</xml_diff>

<commit_message>
Practice 3Sum & 3Sum Closest
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="224">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -63,6 +63,24 @@
     <t xml:space="preserve">https://leetcode.com/problems/pascals-triangle-ii/</t>
   </si>
   <si>
+    <t xml:space="preserve">3Sum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/3sum/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://youtu.be/rM9EthMlXnw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3Sum Closest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/3sum-closest/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pattern</t>
   </si>
   <si>
@@ -105,16 +123,10 @@
     <t xml:space="preserve">167. Two Sum II - Input Array Is Sorted</t>
   </si>
   <si>
-    <t xml:space="preserve">Medium</t>
-  </si>
-  <si>
     <t xml:space="preserve">https://leetcode.com/problems/two-sum-ii-input-array-is-sorted/description/</t>
   </si>
   <si>
     <t xml:space="preserve">15. 3Sum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/3sum/</t>
   </si>
   <si>
     <t xml:space="preserve">19. Remove Nth Node From End of List 
@@ -1540,7 +1552,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="16.15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.78"/>
@@ -1603,11 +1615,49 @@
         <v>11</v>
       </c>
     </row>
+    <row r="4" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="D2" r:id="rId1" display="https://leetcode.com/problems/pascals-triangle/"/>
     <hyperlink ref="E2" r:id="rId2" display="https://youtu.be/ELo7RR-Isjk?si=4BAHl-pa8-hBILgE"/>
     <hyperlink ref="D3" r:id="rId3" display="https://leetcode.com/problems/pascals-triangle-ii/"/>
+    <hyperlink ref="D4" r:id="rId4" display="https://leetcode.com/problems/3sum/"/>
+    <hyperlink ref="E4" r:id="rId5" display="https://youtu.be/rM9EthMlXnw"/>
+    <hyperlink ref="D5" r:id="rId6" display="https://leetcode.com/problems/3sum-closest/"/>
+    <hyperlink ref="E5" r:id="rId7" display="https://youtu.be/rM9EthMlXnw"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -1642,7 +1692,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>1</v>
@@ -1654,10 +1704,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1665,19 +1715,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="D2" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G2" s="8" t="n">
         <v>3</v>
@@ -1688,19 +1738,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D3" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G3" s="8" t="n">
         <v>2</v>
@@ -1711,19 +1761,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="D4" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G4" s="8" t="n">
         <v>3</v>
@@ -1734,19 +1784,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="9" t="s">
         <v>24</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>18</v>
       </c>
       <c r="G5" s="8" t="n">
         <v>3</v>
@@ -1757,19 +1807,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G6" s="8" t="n">
         <v>3</v>
@@ -1780,19 +1830,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G7" s="8" t="n">
         <v>3</v>
@@ -1803,19 +1853,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G8" s="8" t="n">
         <v>4</v>
@@ -1826,19 +1876,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G9" s="8" t="n">
         <v>4</v>
@@ -1849,19 +1899,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G10" s="8" t="n">
         <v>6</v>
@@ -1872,19 +1922,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G11" s="8" t="n">
         <v>6</v>
@@ -1895,19 +1945,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G12" s="8" t="n">
         <v>6</v>
@@ -1918,16 +1968,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C13" s="12" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="F13" s="12"/>
       <c r="G13" s="14"/>
@@ -1937,16 +1987,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C14" s="12" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F14" s="12"/>
       <c r="G14" s="14"/>
@@ -1956,16 +2006,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C15" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="D15" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="12" t="s">
-        <v>41</v>
-      </c>
       <c r="E15" s="13" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F15" s="12"/>
       <c r="G15" s="14"/>
@@ -1975,16 +2025,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C16" s="12" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F16" s="12"/>
       <c r="G16" s="14"/>
@@ -1994,19 +2044,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="15" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="F17" s="15" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G17" s="17" t="n">
         <v>2</v>
@@ -2017,19 +2067,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G18" s="8" t="n">
         <v>5</v>
@@ -2040,22 +2090,22 @@
         <v>18</v>
       </c>
       <c r="B19" s="15" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E19" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="F19" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="F19" s="18" t="s">
-        <v>52</v>
-      </c>
       <c r="G19" s="20" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2063,19 +2113,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G20" s="8" t="n">
         <v>5</v>
@@ -2086,22 +2136,22 @@
         <v>20</v>
       </c>
       <c r="B21" s="15" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E21" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G21" s="20" t="s">
         <v>61</v>
-      </c>
-      <c r="F21" s="18" t="s">
-        <v>52</v>
-      </c>
-      <c r="G21" s="20" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2109,19 +2159,19 @@
         <v>21</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G22" s="8" t="n">
         <v>5</v>
@@ -2132,19 +2182,19 @@
         <v>22</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D23" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G23" s="8" t="n">
         <v>2</v>
@@ -2155,19 +2205,19 @@
         <v>23</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D24" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G24" s="8" t="n">
         <v>2</v>
@@ -2178,19 +2228,19 @@
         <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>7</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G25" s="8" t="n">
         <v>2</v>
@@ -2201,19 +2251,19 @@
         <v>25</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G26" s="8" t="n">
         <v>4</v>
@@ -2253,7 +2303,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C1" s="23" t="s">
         <v>1</v>
@@ -2265,10 +2315,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G1" s="24" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2276,19 +2326,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="26" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D2" s="26" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="27" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F2" s="26" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G2" s="28" t="n">
         <v>8</v>
@@ -2299,19 +2349,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="26" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D3" s="26" t="s">
         <v>7</v>
       </c>
       <c r="E3" s="27" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F3" s="26" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G3" s="28" t="n">
         <v>8</v>
@@ -2322,19 +2372,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D4" s="26" t="s">
         <v>7</v>
       </c>
       <c r="E4" s="27" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F4" s="26" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G4" s="28" t="n">
         <v>8</v>
@@ -2345,19 +2395,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="30" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C5" s="30" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D5" s="30" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E5" s="31" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F5" s="30" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G5" s="32" t="n">
         <v>11</v>
@@ -2368,19 +2418,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C6" s="26" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D6" s="26" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E6" s="27" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="F6" s="26" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G6" s="28" t="n">
         <v>9</v>
@@ -2391,19 +2441,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C7" s="26" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D7" s="26" t="s">
         <v>7</v>
       </c>
       <c r="E7" s="27" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F7" s="26" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G7" s="28" t="n">
         <v>9</v>
@@ -2414,19 +2464,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C8" s="26" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D8" s="26" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E8" s="27" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F8" s="26" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G8" s="28" t="n">
         <v>10</v>
@@ -2437,22 +2487,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="D9" s="33" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E9" s="35" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F9" s="34" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G9" s="36" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="29.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2460,19 +2510,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E10" s="27" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F10" s="26" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G10" s="28" t="n">
         <v>8</v>
@@ -2483,19 +2533,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C11" s="26" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D11" s="26" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E11" s="27" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="F11" s="26" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G11" s="28" t="n">
         <v>8</v>
@@ -2506,19 +2556,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E12" s="27" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="F12" s="26" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G12" s="28" t="n">
         <v>9</v>
@@ -2583,7 +2633,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="39" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C1" s="39" t="s">
         <v>1</v>
@@ -2595,10 +2645,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="39" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G1" s="40" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="27.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2606,19 +2656,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C2" s="42" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D2" s="42" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E2" s="43" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F2" s="42" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G2" s="44" t="n">
         <v>15</v>
@@ -2629,16 +2679,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="45" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C3" s="45" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D3" s="45" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E3" s="46" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="F3" s="45"/>
       <c r="G3" s="45"/>
@@ -2648,16 +2698,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="47" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C4" s="47" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D4" s="47" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E4" s="48" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="F4" s="47"/>
       <c r="G4" s="47"/>
@@ -2667,19 +2717,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D5" s="42" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E5" s="43" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="F5" s="42" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="G5" s="44" t="n">
         <v>18</v>
@@ -2690,16 +2740,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="49" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C6" s="49" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D6" s="49" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E6" s="50" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="F6" s="49"/>
       <c r="G6" s="49"/>
@@ -2709,19 +2759,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C7" s="42" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D7" s="42" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E7" s="43" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="F7" s="42" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G7" s="44" t="n">
         <v>14</v>
@@ -2732,19 +2782,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C8" s="42" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="D8" s="42" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E8" s="43" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="F8" s="42" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G8" s="44" t="n">
         <v>13</v>
@@ -2755,19 +2805,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C9" s="42" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="D9" s="42" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="43" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F9" s="42" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G9" s="44" t="n">
         <v>14</v>
@@ -2778,16 +2828,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C10" s="42" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D10" s="42" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="E10" s="43" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="F10" s="42"/>
       <c r="G10" s="44"/>
@@ -2797,19 +2847,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C11" s="42" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="D11" s="42" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E11" s="43" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F11" s="42" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G11" s="44" t="n">
         <v>16</v>
@@ -2820,19 +2870,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C12" s="42" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="D12" s="42" t="s">
         <v>7</v>
       </c>
       <c r="E12" s="43" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="F12" s="42" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G12" s="44" t="n">
         <v>14</v>
@@ -2843,19 +2893,19 @@
         <v>12</v>
       </c>
       <c r="B13" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C13" s="42" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D13" s="42" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E13" s="43" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="F13" s="42" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G13" s="44" t="n">
         <v>17</v>
@@ -2866,16 +2916,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="49" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C14" s="49" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D14" s="49" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E14" s="50" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="F14" s="49"/>
       <c r="G14" s="49"/>
@@ -2885,16 +2935,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C15" s="49" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="D15" s="49" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E15" s="50" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="F15" s="49"/>
       <c r="G15" s="49"/>
@@ -2904,16 +2954,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="45" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C16" s="45" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="D16" s="45" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E16" s="46" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F16" s="45"/>
       <c r="G16" s="49"/>
@@ -2923,19 +2973,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C17" s="42" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D17" s="42" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E17" s="43" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="F17" s="42" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G17" s="44" t="n">
         <v>13</v>
@@ -2946,19 +2996,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C18" s="42" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="D18" s="42" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E18" s="43" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="F18" s="42" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G18" s="44" t="n">
         <v>13</v>
@@ -2969,16 +3019,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C19" s="42" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D19" s="42" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E19" s="43" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="F19" s="42"/>
       <c r="G19" s="44"/>
@@ -2988,16 +3038,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="42" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C20" s="42" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D20" s="42" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="E20" s="43" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="F20" s="42"/>
       <c r="G20" s="44"/>
@@ -3062,7 +3112,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>1</v>
@@ -3074,10 +3124,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>5</v>
@@ -3107,19 +3157,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C2" s="54" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="D2" s="54" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E2" s="55" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F2" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G2" s="54" t="n">
         <v>21</v>
@@ -3150,19 +3200,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C3" s="54" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="D3" s="54" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E3" s="55" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F3" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G3" s="54" t="n">
         <v>23</v>
@@ -3193,19 +3243,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C4" s="54" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D4" s="54" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E4" s="55" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="F4" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G4" s="54" t="n">
         <v>22</v>
@@ -3236,21 +3286,21 @@
         <v>4</v>
       </c>
       <c r="B5" s="57" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C5" s="58" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="D5" s="56" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E5" s="59" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="F5" s="58"/>
       <c r="G5" s="58"/>
       <c r="H5" s="58" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
@@ -3277,19 +3327,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C6" s="54" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D6" s="54" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E6" s="55" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="F6" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G6" s="54" t="n">
         <v>22</v>
@@ -3320,25 +3370,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C7" s="54" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D7" s="54" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E7" s="55" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F7" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G7" s="54" t="n">
         <v>24</v>
       </c>
       <c r="H7" s="54" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
@@ -3365,25 +3415,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C8" s="54" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D8" s="54" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E8" s="55" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F8" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G8" s="54" t="n">
         <v>28</v>
       </c>
       <c r="H8" s="54" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
@@ -3410,25 +3460,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C9" s="54" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D9" s="54" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E9" s="55" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F9" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G9" s="54" t="n">
         <v>30</v>
       </c>
       <c r="H9" s="54" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
@@ -3455,25 +3505,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C10" s="54" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D10" s="52" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E10" s="55" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F10" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G10" s="54" t="n">
         <v>29</v>
       </c>
       <c r="H10" s="54" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
@@ -3500,19 +3550,19 @@
         <v>10</v>
       </c>
       <c r="B11" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C11" s="54" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="D11" s="54" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E11" s="55" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F11" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G11" s="54" t="n">
         <v>21</v>
@@ -3543,16 +3593,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C12" s="54" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="D12" s="54" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E12" s="55" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="F12" s="54"/>
       <c r="G12" s="54"/>
@@ -3582,16 +3632,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C13" s="54" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D13" s="54" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E13" s="55" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="F13" s="54"/>
       <c r="G13" s="54"/>
@@ -3621,23 +3671,23 @@
         <v>13</v>
       </c>
       <c r="B14" s="61" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C14" s="62" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="D14" s="62" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E14" s="63"/>
       <c r="F14" s="64" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G14" s="64" t="n">
         <v>25</v>
       </c>
       <c r="H14" s="64" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="I14" s="5"/>
       <c r="J14" s="5"/>
@@ -3664,23 +3714,23 @@
         <v>14</v>
       </c>
       <c r="B15" s="61" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C15" s="62" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D15" s="62" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E15" s="63"/>
       <c r="F15" s="64" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G15" s="64" t="n">
         <v>25</v>
       </c>
       <c r="H15" s="64" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="I15" s="5"/>
       <c r="J15" s="5"/>
@@ -3707,25 +3757,25 @@
         <v>15</v>
       </c>
       <c r="B16" s="61" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C16" s="62" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="D16" s="62" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E16" s="63" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="F16" s="64" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G16" s="64" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="H16" s="64" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="I16" s="5"/>
       <c r="J16" s="5"/>
@@ -3752,25 +3802,25 @@
         <v>16</v>
       </c>
       <c r="B17" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C17" s="54" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="D17" s="52" t="s">
         <v>7</v>
       </c>
       <c r="E17" s="55" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="F17" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G17" s="54" t="n">
         <v>27</v>
       </c>
       <c r="H17" s="64" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="I17" s="5"/>
       <c r="J17" s="5"/>
@@ -3797,25 +3847,25 @@
         <v>17</v>
       </c>
       <c r="B18" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C18" s="54" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="D18" s="52" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E18" s="55" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F18" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G18" s="54" t="n">
         <v>27</v>
       </c>
       <c r="H18" s="64" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="I18" s="5"/>
       <c r="J18" s="5"/>
@@ -3842,25 +3892,25 @@
         <v>18</v>
       </c>
       <c r="B19" s="53" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C19" s="54" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="D19" s="52" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E19" s="55" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="F19" s="54" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G19" s="54" t="n">
         <v>29</v>
       </c>
       <c r="H19" s="64" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
@@ -3887,25 +3937,25 @@
         <v>19</v>
       </c>
       <c r="B20" s="66" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C20" s="67" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="D20" s="68" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E20" s="69" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="F20" s="67" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G20" s="67" t="n">
         <v>27</v>
       </c>
       <c r="H20" s="67" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
@@ -3932,16 +3982,16 @@
         <v>20</v>
       </c>
       <c r="B21" s="66" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C21" s="67" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="D21" s="68" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E21" s="69" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F21" s="67"/>
       <c r="G21" s="67"/>
@@ -3971,16 +4021,16 @@
         <v>21</v>
       </c>
       <c r="B22" s="66" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C22" s="67" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="D22" s="68" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E22" s="69" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="F22" s="67"/>
       <c r="G22" s="67"/>
@@ -4010,16 +4060,16 @@
         <v>22</v>
       </c>
       <c r="B23" s="66" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C23" s="67" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="D23" s="67" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E23" s="69" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="F23" s="67"/>
       <c r="G23" s="67"/>
@@ -18166,7 +18216,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -18178,10 +18228,10 @@
         <v>3</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="G1" s="71" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="H1" s="71" t="s">
         <v>5</v>
@@ -18192,25 +18242,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C2" s="72" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D2" s="72" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="73" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="F2" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G2" s="64" t="n">
         <v>32</v>
       </c>
       <c r="H2" s="64" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18218,19 +18268,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C3" s="72" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="D3" s="72" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="E3" s="73" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="F3" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G3" s="64" t="n">
         <v>36</v>
@@ -18242,25 +18292,25 @@
         <v>3</v>
       </c>
       <c r="B4" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C4" s="72" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="D4" s="72" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E4" s="73" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="F4" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G4" s="64" t="n">
         <v>33</v>
       </c>
       <c r="H4" s="64" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18268,25 +18318,25 @@
         <v>4</v>
       </c>
       <c r="B5" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C5" s="72" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="D5" s="72" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E5" s="73" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="F5" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G5" s="64" t="n">
         <v>33</v>
       </c>
       <c r="H5" s="64" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18294,25 +18344,25 @@
         <v>5</v>
       </c>
       <c r="B6" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C6" s="72" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="D6" s="72" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E6" s="73" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="F6" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G6" s="64" t="n">
         <v>34</v>
       </c>
       <c r="H6" s="64" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18320,25 +18370,25 @@
         <v>6</v>
       </c>
       <c r="B7" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C7" s="72" t="s">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="D7" s="72" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E7" s="73" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="F7" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G7" s="64" t="n">
         <v>37</v>
       </c>
       <c r="H7" s="64" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18346,25 +18396,25 @@
         <v>7</v>
       </c>
       <c r="B8" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C8" s="72" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="D8" s="72" t="s">
         <v>7</v>
       </c>
       <c r="E8" s="73" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="F8" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G8" s="64" t="n">
         <v>32</v>
       </c>
       <c r="H8" s="64" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18372,25 +18422,25 @@
         <v>8</v>
       </c>
       <c r="B9" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C9" s="72" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="D9" s="72" t="s">
         <v>7</v>
       </c>
       <c r="E9" s="73" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="F9" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G9" s="64" t="n">
         <v>32</v>
       </c>
       <c r="H9" s="64" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18398,25 +18448,25 @@
         <v>9</v>
       </c>
       <c r="B10" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C10" s="72" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="D10" s="72" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E10" s="73" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="F10" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G10" s="64" t="n">
         <v>35</v>
       </c>
       <c r="H10" s="64" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18424,25 +18474,25 @@
         <v>10</v>
       </c>
       <c r="B11" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C11" s="72" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="D11" s="72" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E11" s="73" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="F11" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G11" s="64" t="n">
         <v>37</v>
       </c>
       <c r="H11" s="64" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18450,23 +18500,23 @@
         <v>11</v>
       </c>
       <c r="B12" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C12" s="72" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="D12" s="72" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="E12" s="73" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="F12" s="74"/>
       <c r="G12" s="64" t="n">
         <v>38</v>
       </c>
       <c r="H12" s="64" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18474,25 +18524,25 @@
         <v>12</v>
       </c>
       <c r="B13" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C13" s="72" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="D13" s="72" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E13" s="73" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="F13" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G13" s="64" t="n">
         <v>34</v>
       </c>
       <c r="H13" s="64" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="26.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -18500,19 +18550,19 @@
         <v>13</v>
       </c>
       <c r="B14" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C14" s="72" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="D14" s="72" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E14" s="73" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="F14" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G14" s="64" t="n">
         <v>35</v>
@@ -18524,17 +18574,17 @@
         <v>14</v>
       </c>
       <c r="B15" s="72" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="C15" s="72" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="D15" s="72" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="E15" s="74"/>
       <c r="F15" s="74" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G15" s="64" t="n">
         <v>32</v>

</xml_diff>

<commit_message>
Start with Heaps Pattern - Day 39
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Practice Problems (Kunal + Anuj" sheetId="1" state="visible" r:id="rId3"/>
@@ -14,6 +14,7 @@
     <sheet name="Sliding Window" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="Intervals" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Linked List - In-Place Manipula" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Heaps" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="257">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -711,6 +712,93 @@
   </si>
   <si>
     <t xml:space="preserve">Dummy Node Concept (Theory)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Heaps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">502. IPO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/ipo/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">295. Find Median from Data Stream</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/find-median-from-data-stream/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">480. Sliding Window Median</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hard (BFA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/sliding-window-median/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">621. Task Scheduler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/task-scheduler/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2402. Meeting Rooms III</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/meeting-rooms-iii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2231. Largest Number After Digit Swaps by Parity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/largest-number-after-digit-swaps-by-parity/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">436. Find Right Interval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/find-right-interval/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minimum Cost of ropes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.geeksforgeeks.org/problems/minimum-cost-of-ropes-1587115620/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1405. Longest Happy String</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/longest-happy-string/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1792. Maximum Average Pass Ratio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/maximum-average-pass-ratio/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1942. The Number of the Smallest Unoccupied Chair</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/the-number-of-the-smallest-unoccupied-chair/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1354. Construct Target Array With Multiple Sums</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/construct-target-array-with-multiple-sums/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1046. Last Stone Weight</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/last-stone-weight/description/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hard (Optimised)</t>
   </si>
 </sst>
 </file>
@@ -1014,7 +1102,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1319,6 +1407,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18653,4 +18745,314 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="16.15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="71" width="5.31"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="71" width="11.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="71" width="64.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="71" width="19.77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="71" width="69.19"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="71" width="11.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="71" width="10.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="71" width="33.24"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="71" width="11.55"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="76" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="76" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="76" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="76" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="76" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="76" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="72" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="72" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>235</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" display="https://leetcode.com/problems/ipo/"/>
+    <hyperlink ref="E3" r:id="rId2" display="https://leetcode.com/problems/find-median-from-data-stream/"/>
+    <hyperlink ref="E4" r:id="rId3" display="https://leetcode.com/problems/sliding-window-median/"/>
+    <hyperlink ref="E5" r:id="rId4" display="https://leetcode.com/problems/task-scheduler/"/>
+    <hyperlink ref="E6" r:id="rId5" display="https://leetcode.com/problems/meeting-rooms-iii/"/>
+    <hyperlink ref="E7" r:id="rId6" display="https://leetcode.com/problems/largest-number-after-digit-swaps-by-parity/"/>
+    <hyperlink ref="E8" r:id="rId7" display="https://leetcode.com/problems/find-right-interval/"/>
+    <hyperlink ref="E9" r:id="rId8" display="https://www.geeksforgeeks.org/problems/minimum-cost-of-ropes-1587115620/1"/>
+    <hyperlink ref="E10" r:id="rId9" display="https://leetcode.com/problems/longest-happy-string/"/>
+    <hyperlink ref="E11" r:id="rId10" display="https://leetcode.com/problems/maximum-average-pass-ratio/"/>
+    <hyperlink ref="E12" r:id="rId11" display="https://leetcode.com/problems/the-number-of-the-smallest-unoccupied-chair/"/>
+    <hyperlink ref="E13" r:id="rId12" display="https://leetcode.com/problems/construct-target-array-with-multiple-sums/"/>
+    <hyperlink ref="E14" r:id="rId13" display="https://leetcode.com/problems/last-stone-weight/description/"/>
+    <hyperlink ref="E15" r:id="rId14" display="https://leetcode.com/problems/sliding-window-median/"/>
+  </hyperlinks>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Done with day 41
</commit_message>
<xml_diff>
--- a/2.Patterns Practice.xlsx
+++ b/2.Patterns Practice.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="244">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -711,6 +711,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/largest-number-after-digit-swaps-by-parity/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Learn about java conversion methods: int → String → char[] and back to int</t>
   </si>
   <si>
     <t xml:space="preserve">436. Find Right Interval</t>
@@ -1360,11 +1363,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -18575,27 +18578,27 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="69" width="69.19"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="6" min="6" style="69" width="11.55"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="69" width="10.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="69" width="33.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="75" width="44.23"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="69" width="11.55"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="75" t="s">
+      <c r="B1" s="76" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="75" t="s">
+      <c r="C1" s="76" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="75" t="s">
+      <c r="D1" s="76" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="75" t="s">
+      <c r="E1" s="76" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="75" t="s">
+      <c r="F1" s="76" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="71" t="s">
@@ -18606,240 +18609,255 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="76" t="n">
+      <c r="A2" s="75" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="76" t="s">
+      <c r="B2" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C2" s="76" t="s">
+      <c r="C2" s="75" t="s">
         <v>215</v>
       </c>
-      <c r="D2" s="76" t="s">
+      <c r="D2" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="E2" s="76" t="s">
+      <c r="E2" s="75" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="76" t="n">
+      <c r="A3" s="75" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="76" t="s">
+      <c r="B3" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C3" s="76" t="s">
+      <c r="C3" s="75" t="s">
         <v>217</v>
       </c>
-      <c r="D3" s="76" t="s">
+      <c r="D3" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="76" t="s">
+      <c r="E3" s="75" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="76" t="n">
+      <c r="A4" s="75" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="76" t="s">
+      <c r="B4" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C4" s="76" t="s">
+      <c r="C4" s="75" t="s">
         <v>219</v>
       </c>
-      <c r="D4" s="76" t="s">
+      <c r="D4" s="75" t="s">
         <v>220</v>
       </c>
-      <c r="E4" s="76" t="s">
+      <c r="E4" s="75" t="s">
         <v>221</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="76" t="n">
+      <c r="A5" s="75" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="76" t="s">
+      <c r="B5" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C5" s="76" t="s">
+      <c r="C5" s="75" t="s">
         <v>222</v>
       </c>
-      <c r="D5" s="76" t="s">
+      <c r="D5" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="76" t="s">
+      <c r="E5" s="75" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="76" t="n">
+      <c r="A6" s="75" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="76" t="s">
+      <c r="B6" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C6" s="76" t="s">
+      <c r="C6" s="75" t="s">
         <v>224</v>
       </c>
-      <c r="D6" s="76" t="s">
+      <c r="D6" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="E6" s="76" t="s">
+      <c r="E6" s="75" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="76" t="n">
+    <row r="7" customFormat="false" ht="37.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="75" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="76" t="s">
+      <c r="B7" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C7" s="76" t="s">
+      <c r="C7" s="75" t="s">
         <v>226</v>
       </c>
-      <c r="D7" s="76" t="s">
+      <c r="D7" s="75" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="76" t="s">
+      <c r="E7" s="75" t="s">
         <v>227</v>
       </c>
+      <c r="F7" s="69" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="69" t="n">
+        <v>41</v>
+      </c>
+      <c r="H7" s="75" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="76" t="n">
+      <c r="A8" s="75" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="76" t="s">
+      <c r="B8" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C8" s="76" t="s">
-        <v>228</v>
-      </c>
-      <c r="D8" s="76" t="s">
+      <c r="C8" s="75" t="s">
+        <v>229</v>
+      </c>
+      <c r="D8" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="76" t="s">
-        <v>229</v>
+      <c r="E8" s="75" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="76" t="n">
+      <c r="A9" s="75" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="76" t="s">
+      <c r="B9" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C9" s="76" t="s">
-        <v>230</v>
-      </c>
-      <c r="D9" s="76" t="s">
+      <c r="C9" s="75" t="s">
+        <v>231</v>
+      </c>
+      <c r="D9" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="76" t="s">
-        <v>231</v>
+      <c r="E9" s="75" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="76" t="n">
+      <c r="A10" s="75" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="76" t="s">
+      <c r="B10" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C10" s="76" t="s">
-        <v>232</v>
-      </c>
-      <c r="D10" s="76" t="s">
+      <c r="C10" s="75" t="s">
+        <v>233</v>
+      </c>
+      <c r="D10" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="76" t="s">
-        <v>233</v>
+      <c r="E10" s="75" t="s">
+        <v>234</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="76" t="n">
+      <c r="A11" s="75" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="76" t="s">
+      <c r="B11" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C11" s="76" t="s">
-        <v>234</v>
-      </c>
-      <c r="D11" s="76" t="s">
+      <c r="C11" s="75" t="s">
+        <v>235</v>
+      </c>
+      <c r="D11" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="76" t="s">
-        <v>235</v>
+      <c r="E11" s="75" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="76" t="n">
+      <c r="A12" s="75" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="76" t="s">
+      <c r="B12" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C12" s="76" t="s">
-        <v>236</v>
-      </c>
-      <c r="D12" s="76" t="s">
+      <c r="C12" s="75" t="s">
+        <v>237</v>
+      </c>
+      <c r="D12" s="75" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="76" t="s">
-        <v>237</v>
+      <c r="E12" s="75" t="s">
+        <v>238</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="76" t="n">
+      <c r="A13" s="75" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="76" t="s">
+      <c r="B13" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C13" s="76" t="s">
-        <v>238</v>
-      </c>
-      <c r="D13" s="76" t="s">
+      <c r="C13" s="75" t="s">
+        <v>239</v>
+      </c>
+      <c r="D13" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="E13" s="76" t="s">
-        <v>239</v>
+      <c r="E13" s="75" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="76" t="n">
+      <c r="A14" s="75" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="76" t="s">
+      <c r="B14" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C14" s="76" t="s">
-        <v>240</v>
-      </c>
-      <c r="D14" s="76" t="s">
+      <c r="C14" s="75" t="s">
+        <v>241</v>
+      </c>
+      <c r="D14" s="75" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="76" t="s">
-        <v>241</v>
+      <c r="E14" s="75" t="s">
+        <v>242</v>
+      </c>
+      <c r="F14" s="69" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="69" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="19.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="76" t="n">
+      <c r="A15" s="75" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="76" t="s">
+      <c r="B15" s="75" t="s">
         <v>214</v>
       </c>
-      <c r="C15" s="76" t="s">
+      <c r="C15" s="75" t="s">
         <v>219</v>
       </c>
-      <c r="D15" s="76" t="s">
-        <v>242</v>
-      </c>
-      <c r="E15" s="76" t="s">
+      <c r="D15" s="75" t="s">
+        <v>243</v>
+      </c>
+      <c r="E15" s="75" t="s">
         <v>221</v>
       </c>
     </row>

</xml_diff>